<commit_message>
updated the requirements, as well as updating the print logic
</commit_message>
<xml_diff>
--- a/core/main/templates/print_excel/cmf_template.xlsx
+++ b/core/main/templates/print_excel/cmf_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brant\VS Code Web\ColorMatch\core\main\templates\print_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6384B01-B8CB-4C49-8ABA-E76EDE5497ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{840B428F-DF6C-4563-8BC3-A84843E4ADA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -386,44 +386,6 @@
       </extLst>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -431,13 +393,51 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -978,8 +978,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7087604" y="6750220"/>
-          <a:ext cx="824" cy="444248"/>
+          <a:off x="8253984" y="10088300"/>
+          <a:ext cx="824" cy="581927"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -1461,105 +1461,105 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22"/>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
+      <c r="A1" s="29"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="22"/>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
+      <c r="A2" s="29"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="29"/>
+      <c r="O2" s="29"/>
+      <c r="P2" s="29"/>
+      <c r="Q2" s="29"/>
     </row>
     <row r="3" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="22"/>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="33" t="s">
+      <c r="A3" s="29"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="N3" s="33"/>
-      <c r="O3" s="33"/>
-      <c r="P3" s="33"/>
-      <c r="Q3" s="22"/>
+      <c r="N3" s="31"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="29"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="22"/>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
+      <c r="A4" s="29"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="29"/>
+      <c r="M4" s="29"/>
+      <c r="N4" s="29"/>
+      <c r="O4" s="29"/>
+      <c r="P4" s="29"/>
+      <c r="Q4" s="29"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="22"/>
-      <c r="B5" s="22"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
+      <c r="A5" s="29"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="29"/>
+      <c r="M5" s="29"/>
+      <c r="N5" s="29"/>
+      <c r="O5" s="29"/>
+      <c r="P5" s="29"/>
+      <c r="Q5" s="29"/>
     </row>
     <row r="6" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
-      <c r="B6" s="22"/>
+      <c r="A6" s="29"/>
+      <c r="B6" s="29"/>
       <c r="C6" s="1" t="s">
         <v>35</v>
       </c>
@@ -1573,16 +1573,16 @@
       <c r="I6" s="25"/>
       <c r="J6" s="25"/>
       <c r="K6" s="1"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="22"/>
-      <c r="Q6" s="22"/>
+      <c r="L6" s="29"/>
+      <c r="M6" s="29"/>
+      <c r="N6" s="29"/>
+      <c r="O6" s="29"/>
+      <c r="P6" s="29"/>
+      <c r="Q6" s="29"/>
     </row>
     <row r="7" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="22"/>
-      <c r="B7" s="22"/>
+      <c r="A7" s="29"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="6" t="s">
         <v>1</v>
       </c>
@@ -1590,22 +1590,22 @@
       <c r="E7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="31"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="31"/>
-      <c r="I7" s="31"/>
-      <c r="J7" s="31"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
       <c r="K7" s="13"/>
       <c r="L7" s="10"/>
       <c r="M7" s="10"/>
       <c r="N7" s="10"/>
       <c r="O7" s="10"/>
       <c r="P7" s="1"/>
-      <c r="Q7" s="22"/>
+      <c r="Q7" s="29"/>
     </row>
     <row r="8" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="22"/>
-      <c r="B8" s="22"/>
+      <c r="A8" s="29"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="6" t="s">
         <v>2</v>
       </c>
@@ -1613,17 +1613,17 @@
       <c r="E8" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="29"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="35"/>
       <c r="K8" s="17"/>
-      <c r="Q8" s="22"/>
+      <c r="Q8" s="29"/>
     </row>
     <row r="9" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="22"/>
-      <c r="B9" s="22"/>
+      <c r="A9" s="29"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="6" t="s">
         <v>40</v>
       </c>
@@ -1631,31 +1631,31 @@
       <c r="E9" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="29"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
+      <c r="J9" s="35"/>
       <c r="K9" s="17"/>
-      <c r="Q9" s="22"/>
+      <c r="Q9" s="29"/>
     </row>
     <row r="10" spans="1:17" ht="3.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="22"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
+      <c r="A10" s="29"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
       <c r="K10" s="12"/>
-      <c r="Q10" s="22"/>
+      <c r="Q10" s="29"/>
     </row>
     <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="22"/>
-      <c r="B11" s="22"/>
+      <c r="A11" s="29"/>
+      <c r="B11" s="29"/>
       <c r="C11" s="6" t="s">
         <v>3</v>
       </c>
@@ -1674,11 +1674,11 @@
         <v>9</v>
       </c>
       <c r="K11" s="1"/>
-      <c r="Q11" s="22"/>
+      <c r="Q11" s="29"/>
     </row>
     <row r="12" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
-      <c r="B12" s="22"/>
+      <c r="A12" s="29"/>
+      <c r="B12" s="29"/>
       <c r="C12" s="6" t="s">
         <v>5</v>
       </c>
@@ -1686,22 +1686,22 @@
       <c r="E12" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36"/>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
       <c r="K12" s="13"/>
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
       <c r="O12" s="10"/>
       <c r="P12" s="1"/>
-      <c r="Q12" s="22"/>
+      <c r="Q12" s="29"/>
     </row>
     <row r="13" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="22"/>
-      <c r="B13" s="22"/>
+      <c r="A13" s="29"/>
+      <c r="B13" s="29"/>
       <c r="C13" s="6" t="s">
         <v>6</v>
       </c>
@@ -1709,22 +1709,22 @@
       <c r="E13" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F13" s="31"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="31"/>
-      <c r="I13" s="31"/>
-      <c r="J13" s="31"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
       <c r="K13" s="14"/>
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
       <c r="N13" s="11"/>
       <c r="O13" s="11"/>
       <c r="P13" s="1"/>
-      <c r="Q13" s="22"/>
+      <c r="Q13" s="29"/>
     </row>
     <row r="14" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="22"/>
-      <c r="B14" s="22"/>
+      <c r="A14" s="29"/>
+      <c r="B14" s="29"/>
       <c r="C14" s="6" t="s">
         <v>7</v>
       </c>
@@ -1732,60 +1732,60 @@
       <c r="E14" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="34"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="34"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
       <c r="K14" s="10"/>
       <c r="L14" s="10"/>
       <c r="M14" s="10"/>
       <c r="N14" s="10"/>
       <c r="O14" s="10"/>
       <c r="P14" s="1"/>
-      <c r="Q14" s="22"/>
+      <c r="Q14" s="29"/>
     </row>
     <row r="15" spans="1:17" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="22"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="22"/>
-      <c r="L15" s="22"/>
-      <c r="M15" s="22"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="22"/>
-      <c r="P15" s="22"/>
-      <c r="Q15" s="22"/>
+      <c r="A15" s="29"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
+      <c r="I15" s="29"/>
+      <c r="J15" s="29"/>
+      <c r="K15" s="29"/>
+      <c r="L15" s="29"/>
+      <c r="M15" s="29"/>
+      <c r="N15" s="29"/>
+      <c r="O15" s="29"/>
+      <c r="P15" s="29"/>
+      <c r="Q15" s="29"/>
     </row>
     <row r="16" spans="1:17" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="22"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="22"/>
-      <c r="M16" s="22"/>
-      <c r="N16" s="22"/>
-      <c r="O16" s="22"/>
-      <c r="P16" s="22"/>
-      <c r="Q16" s="22"/>
+      <c r="A16" s="29"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="29"/>
+      <c r="J16" s="29"/>
+      <c r="K16" s="29"/>
+      <c r="L16" s="29"/>
+      <c r="M16" s="29"/>
+      <c r="N16" s="29"/>
+      <c r="O16" s="29"/>
+      <c r="P16" s="29"/>
+      <c r="Q16" s="29"/>
     </row>
     <row r="17" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="22"/>
-      <c r="B17" s="22"/>
+      <c r="A17" s="29"/>
+      <c r="B17" s="29"/>
       <c r="C17" s="6" t="s">
         <v>41</v>
       </c>
@@ -1812,30 +1812,30 @@
       <c r="M17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="Q17" s="22"/>
+      <c r="Q17" s="29"/>
     </row>
     <row r="18" spans="1:17" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="22"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="22"/>
-      <c r="P18" s="22"/>
-      <c r="Q18" s="22"/>
+      <c r="A18" s="29"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="29"/>
+      <c r="I18" s="29"/>
+      <c r="J18" s="29"/>
+      <c r="K18" s="29"/>
+      <c r="L18" s="29"/>
+      <c r="M18" s="29"/>
+      <c r="N18" s="29"/>
+      <c r="O18" s="29"/>
+      <c r="P18" s="29"/>
+      <c r="Q18" s="29"/>
     </row>
     <row r="19" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="22"/>
-      <c r="B19" s="22"/>
+      <c r="A19" s="29"/>
+      <c r="B19" s="29"/>
       <c r="F19" s="16" t="b">
         <v>0</v>
       </c>
@@ -1855,42 +1855,42 @@
       <c r="M19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q19" s="22"/>
+      <c r="Q19" s="29"/>
     </row>
     <row r="20" spans="1:17" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="22"/>
-      <c r="B20" s="22"/>
+      <c r="A20" s="29"/>
+      <c r="B20" s="29"/>
       <c r="G20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
       <c r="M20" s="1"/>
-      <c r="Q20" s="22"/>
+      <c r="Q20" s="29"/>
     </row>
     <row r="21" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="22"/>
-      <c r="B21" s="22"/>
-      <c r="F21" s="36" t="b">
+      <c r="A21" s="29"/>
+      <c r="B21" s="29"/>
+      <c r="F21" s="22" t="b">
         <v>0</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H21" s="32"/>
-      <c r="I21" s="32"/>
-      <c r="J21" s="32"/>
-      <c r="K21" s="32"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="32"/>
-      <c r="N21" s="32"/>
-      <c r="Q21" s="22"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="37"/>
+      <c r="J21" s="37"/>
+      <c r="K21" s="37"/>
+      <c r="L21" s="37"/>
+      <c r="M21" s="37"/>
+      <c r="N21" s="37"/>
+      <c r="Q21" s="29"/>
     </row>
     <row r="22" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="22"/>
-      <c r="B22" s="22"/>
-      <c r="C22" s="37" t="s">
+      <c r="A22" s="29"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="37"/>
+      <c r="D22" s="30"/>
       <c r="E22" s="2" t="s">
         <v>4</v>
       </c>
@@ -1900,39 +1900,39 @@
       <c r="I22" s="25"/>
       <c r="J22" s="25"/>
       <c r="K22" s="1"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="22"/>
-      <c r="O22" s="22"/>
-      <c r="P22" s="22"/>
-      <c r="Q22" s="22"/>
+      <c r="L22" s="29"/>
+      <c r="M22" s="29"/>
+      <c r="N22" s="29"/>
+      <c r="O22" s="29"/>
+      <c r="P22" s="29"/>
+      <c r="Q22" s="29"/>
     </row>
     <row r="23" spans="1:17" ht="4.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="22"/>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="22"/>
-      <c r="N23" s="22"/>
-      <c r="O23" s="22"/>
-      <c r="P23" s="22"/>
-      <c r="Q23" s="22"/>
+      <c r="A23" s="29"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="29"/>
+      <c r="M23" s="29"/>
+      <c r="N23" s="29"/>
+      <c r="O23" s="29"/>
+      <c r="P23" s="29"/>
+      <c r="Q23" s="29"/>
     </row>
     <row r="24" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="22"/>
-      <c r="B24" s="22"/>
-      <c r="C24" s="37" t="s">
+      <c r="A24" s="29"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="D24" s="37"/>
+      <c r="D24" s="30"/>
       <c r="E24" s="2" t="s">
         <v>4</v>
       </c>
@@ -1955,32 +1955,32 @@
       <c r="N24" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="O24" s="22"/>
-      <c r="P24" s="22"/>
-      <c r="Q24" s="22"/>
+      <c r="O24" s="29"/>
+      <c r="P24" s="29"/>
+      <c r="Q24" s="29"/>
     </row>
     <row r="25" spans="1:17" ht="4.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="22"/>
-      <c r="B25" s="22"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="22"/>
-      <c r="J25" s="22"/>
-      <c r="K25" s="22"/>
-      <c r="L25" s="22"/>
-      <c r="M25" s="22"/>
-      <c r="N25" s="22"/>
-      <c r="O25" s="22"/>
-      <c r="P25" s="22"/>
-      <c r="Q25" s="22"/>
+      <c r="A25" s="29"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="29"/>
+      <c r="I25" s="29"/>
+      <c r="J25" s="29"/>
+      <c r="K25" s="29"/>
+      <c r="L25" s="29"/>
+      <c r="M25" s="29"/>
+      <c r="N25" s="29"/>
+      <c r="O25" s="29"/>
+      <c r="P25" s="29"/>
+      <c r="Q25" s="29"/>
     </row>
     <row r="26" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="22"/>
-      <c r="B26" s="22"/>
+      <c r="A26" s="29"/>
+      <c r="B26" s="29"/>
       <c r="F26" s="21" t="b">
         <v>0</v>
       </c>
@@ -1998,27 +1998,27 @@
       <c r="M26" s="25"/>
       <c r="N26" s="25"/>
       <c r="O26" s="25"/>
-      <c r="Q26" s="22"/>
+      <c r="Q26" s="29"/>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A27" s="22"/>
-      <c r="B27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="22"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="22"/>
-      <c r="M27" s="22"/>
-      <c r="N27" s="22"/>
-      <c r="O27" s="22"/>
-      <c r="P27" s="22"/>
-      <c r="Q27" s="22"/>
+      <c r="A27" s="29"/>
+      <c r="B27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="29"/>
+      <c r="I27" s="29"/>
+      <c r="J27" s="29"/>
+      <c r="K27" s="29"/>
+      <c r="L27" s="29"/>
+      <c r="M27" s="29"/>
+      <c r="N27" s="29"/>
+      <c r="O27" s="29"/>
+      <c r="P27" s="29"/>
+      <c r="Q27" s="29"/>
     </row>
     <row r="28" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="22"/>
-      <c r="B28" s="22"/>
+      <c r="A28" s="29"/>
+      <c r="B28" s="29"/>
       <c r="C28" s="6" t="s">
         <v>20</v>
       </c>
@@ -2026,22 +2026,22 @@
       <c r="E28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
-      <c r="J28" s="30"/>
+      <c r="F28" s="36"/>
+      <c r="G28" s="36"/>
+      <c r="H28" s="36"/>
+      <c r="I28" s="36"/>
+      <c r="J28" s="36"/>
       <c r="K28" s="15"/>
       <c r="L28" s="3"/>
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
-      <c r="Q28" s="22"/>
+      <c r="Q28" s="29"/>
     </row>
     <row r="29" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="22"/>
-      <c r="B29" s="22"/>
+      <c r="A29" s="29"/>
+      <c r="B29" s="29"/>
       <c r="C29" s="6" t="s">
         <v>44</v>
       </c>
@@ -2062,18 +2062,18 @@
         <v>22</v>
       </c>
       <c r="K29" s="1"/>
-      <c r="L29" s="23" t="s">
+      <c r="L29" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M29" s="23"/>
-      <c r="N29" s="23"/>
-      <c r="O29" s="23"/>
-      <c r="P29" s="23"/>
-      <c r="Q29" s="22"/>
+      <c r="M29" s="38"/>
+      <c r="N29" s="38"/>
+      <c r="O29" s="38"/>
+      <c r="P29" s="38"/>
+      <c r="Q29" s="29"/>
     </row>
     <row r="30" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="22"/>
-      <c r="B30" s="22"/>
+      <c r="A30" s="29"/>
+      <c r="B30" s="29"/>
       <c r="C30" s="6" t="s">
         <v>45</v>
       </c>
@@ -2081,22 +2081,22 @@
       <c r="E30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="30"/>
-      <c r="J30" s="30"/>
+      <c r="F30" s="36"/>
+      <c r="G30" s="36"/>
+      <c r="H30" s="36"/>
+      <c r="I30" s="36"/>
+      <c r="J30" s="36"/>
       <c r="K30" s="15"/>
-      <c r="L30" s="23"/>
-      <c r="M30" s="23"/>
-      <c r="N30" s="23"/>
-      <c r="O30" s="23"/>
-      <c r="P30" s="23"/>
-      <c r="Q30" s="22"/>
+      <c r="L30" s="38"/>
+      <c r="M30" s="38"/>
+      <c r="N30" s="38"/>
+      <c r="O30" s="38"/>
+      <c r="P30" s="38"/>
+      <c r="Q30" s="29"/>
     </row>
     <row r="31" spans="1:17" ht="21.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="22"/>
-      <c r="B31" s="22"/>
+      <c r="A31" s="29"/>
+      <c r="B31" s="29"/>
       <c r="C31" s="1" t="s">
         <v>31</v>
       </c>
@@ -2117,35 +2117,35 @@
         <v>22</v>
       </c>
       <c r="K31" s="1"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
-      <c r="N31" s="23"/>
-      <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
-      <c r="Q31" s="22"/>
+      <c r="L31" s="38"/>
+      <c r="M31" s="38"/>
+      <c r="N31" s="38"/>
+      <c r="O31" s="38"/>
+      <c r="P31" s="38"/>
+      <c r="Q31" s="29"/>
     </row>
     <row r="32" spans="1:17" ht="4.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="22"/>
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="22"/>
-      <c r="I32" s="22"/>
-      <c r="J32" s="22"/>
-      <c r="K32" s="22"/>
-      <c r="L32" s="22"/>
-      <c r="M32" s="22"/>
-      <c r="N32" s="22"/>
-      <c r="O32" s="22"/>
-      <c r="P32" s="22"/>
-      <c r="Q32" s="22"/>
+      <c r="A32" s="29"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="29"/>
+      <c r="J32" s="29"/>
+      <c r="K32" s="29"/>
+      <c r="L32" s="29"/>
+      <c r="M32" s="29"/>
+      <c r="N32" s="29"/>
+      <c r="O32" s="29"/>
+      <c r="P32" s="29"/>
+      <c r="Q32" s="29"/>
     </row>
     <row r="33" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="22"/>
-      <c r="B33" s="22"/>
+      <c r="A33" s="29"/>
+      <c r="B33" s="29"/>
       <c r="C33" s="6" t="s">
         <v>23</v>
       </c>
@@ -2174,30 +2174,30 @@
       </c>
       <c r="O33" s="25"/>
       <c r="P33" s="25"/>
-      <c r="Q33" s="22"/>
+      <c r="Q33" s="29"/>
     </row>
     <row r="34" spans="1:17" ht="4.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="22"/>
-      <c r="B34" s="22"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22"/>
-      <c r="J34" s="22"/>
-      <c r="K34" s="22"/>
-      <c r="L34" s="22"/>
-      <c r="M34" s="22"/>
-      <c r="N34" s="22"/>
-      <c r="O34" s="22"/>
-      <c r="P34" s="22"/>
-      <c r="Q34" s="22"/>
+      <c r="A34" s="29"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
+      <c r="J34" s="29"/>
+      <c r="K34" s="29"/>
+      <c r="L34" s="29"/>
+      <c r="M34" s="29"/>
+      <c r="N34" s="29"/>
+      <c r="O34" s="29"/>
+      <c r="P34" s="29"/>
+      <c r="Q34" s="29"/>
     </row>
     <row r="35" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="22"/>
-      <c r="B35" s="22"/>
+      <c r="A35" s="29"/>
+      <c r="B35" s="29"/>
       <c r="C35" s="7" t="s">
         <v>36</v>
       </c>
@@ -2205,32 +2205,32 @@
       <c r="E35" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F35" s="35"/>
-      <c r="G35" s="35"/>
-      <c r="H35" s="35"/>
-      <c r="I35" s="35"/>
-      <c r="J35" s="35"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="28"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="28"/>
       <c r="K35" s="18"/>
-      <c r="L35" s="24"/>
-      <c r="M35" s="24"/>
-      <c r="N35" s="24"/>
-      <c r="O35" s="24"/>
-      <c r="P35" s="24"/>
-      <c r="Q35" s="22"/>
+      <c r="L35" s="39"/>
+      <c r="M35" s="39"/>
+      <c r="N35" s="39"/>
+      <c r="O35" s="39"/>
+      <c r="P35" s="39"/>
+      <c r="Q35" s="29"/>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A36" s="22"/>
-      <c r="B36" s="22"/>
-      <c r="L36" s="24"/>
-      <c r="M36" s="24"/>
-      <c r="N36" s="24"/>
-      <c r="O36" s="24"/>
-      <c r="P36" s="24"/>
-      <c r="Q36" s="22"/>
+      <c r="A36" s="29"/>
+      <c r="B36" s="29"/>
+      <c r="L36" s="39"/>
+      <c r="M36" s="39"/>
+      <c r="N36" s="39"/>
+      <c r="O36" s="39"/>
+      <c r="P36" s="39"/>
+      <c r="Q36" s="29"/>
     </row>
     <row r="37" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="22"/>
-      <c r="B37" s="22"/>
+      <c r="A37" s="29"/>
+      <c r="B37" s="29"/>
       <c r="C37" s="1" t="s">
         <v>26</v>
       </c>
@@ -2251,35 +2251,35 @@
         <v>22</v>
       </c>
       <c r="K37" s="1"/>
-      <c r="L37" s="24"/>
-      <c r="M37" s="24"/>
-      <c r="N37" s="24"/>
-      <c r="O37" s="24"/>
-      <c r="P37" s="24"/>
-      <c r="Q37" s="22"/>
+      <c r="L37" s="39"/>
+      <c r="M37" s="39"/>
+      <c r="N37" s="39"/>
+      <c r="O37" s="39"/>
+      <c r="P37" s="39"/>
+      <c r="Q37" s="29"/>
     </row>
     <row r="38" spans="1:17" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="22"/>
-      <c r="B38" s="22"/>
-      <c r="C38" s="22"/>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="22"/>
-      <c r="I38" s="22"/>
-      <c r="J38" s="22"/>
-      <c r="K38" s="22"/>
-      <c r="L38" s="22"/>
-      <c r="M38" s="22"/>
-      <c r="N38" s="22"/>
-      <c r="O38" s="22"/>
-      <c r="P38" s="22"/>
-      <c r="Q38" s="22"/>
+      <c r="A38" s="29"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="29"/>
+      <c r="J38" s="29"/>
+      <c r="K38" s="29"/>
+      <c r="L38" s="29"/>
+      <c r="M38" s="29"/>
+      <c r="N38" s="29"/>
+      <c r="O38" s="29"/>
+      <c r="P38" s="29"/>
+      <c r="Q38" s="29"/>
     </row>
     <row r="39" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" s="22"/>
-      <c r="B39" s="22"/>
+      <c r="A39" s="29"/>
+      <c r="B39" s="29"/>
       <c r="C39" s="6" t="s">
         <v>27</v>
       </c>
@@ -2300,11 +2300,11 @@
         <v>29</v>
       </c>
       <c r="K39" s="1"/>
-      <c r="Q39" s="22"/>
+      <c r="Q39" s="29"/>
     </row>
     <row r="40" spans="1:17" ht="3.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="22"/>
-      <c r="B40" s="22"/>
+      <c r="A40" s="29"/>
+      <c r="B40" s="29"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
@@ -2314,11 +2314,11 @@
       <c r="K40" s="1"/>
       <c r="N40" s="1"/>
       <c r="P40" s="1"/>
-      <c r="Q40" s="22"/>
+      <c r="Q40" s="29"/>
     </row>
     <row r="41" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="22"/>
-      <c r="B41" s="22"/>
+      <c r="A41" s="29"/>
+      <c r="B41" s="29"/>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
@@ -2328,38 +2328,38 @@
       <c r="G41" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H41" s="32"/>
-      <c r="I41" s="32"/>
-      <c r="J41" s="32"/>
-      <c r="K41" s="32"/>
-      <c r="L41" s="32"/>
-      <c r="M41" s="32"/>
+      <c r="H41" s="37"/>
+      <c r="I41" s="37"/>
+      <c r="J41" s="37"/>
+      <c r="K41" s="37"/>
+      <c r="L41" s="37"/>
+      <c r="M41" s="37"/>
       <c r="N41" s="1"/>
       <c r="P41" s="1"/>
-      <c r="Q41" s="22"/>
+      <c r="Q41" s="29"/>
     </row>
     <row r="42" spans="1:17" ht="3.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="22"/>
-      <c r="B42" s="22"/>
-      <c r="C42" s="22"/>
-      <c r="D42" s="22"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="22"/>
-      <c r="I42" s="22"/>
-      <c r="J42" s="22"/>
-      <c r="K42" s="22"/>
-      <c r="L42" s="22"/>
-      <c r="M42" s="22"/>
-      <c r="N42" s="22"/>
-      <c r="O42" s="22"/>
-      <c r="P42" s="22"/>
-      <c r="Q42" s="22"/>
+      <c r="A42" s="29"/>
+      <c r="B42" s="29"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="29"/>
+      <c r="H42" s="29"/>
+      <c r="I42" s="29"/>
+      <c r="J42" s="29"/>
+      <c r="K42" s="29"/>
+      <c r="L42" s="29"/>
+      <c r="M42" s="29"/>
+      <c r="N42" s="29"/>
+      <c r="O42" s="29"/>
+      <c r="P42" s="29"/>
+      <c r="Q42" s="29"/>
     </row>
     <row r="43" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="22"/>
-      <c r="B43" s="22"/>
+      <c r="A43" s="29"/>
+      <c r="B43" s="29"/>
       <c r="C43" s="6" t="s">
         <v>30</v>
       </c>
@@ -2367,22 +2367,22 @@
       <c r="E43" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F43" s="30"/>
-      <c r="G43" s="30"/>
-      <c r="H43" s="30"/>
-      <c r="I43" s="30"/>
-      <c r="J43" s="30"/>
+      <c r="F43" s="36"/>
+      <c r="G43" s="36"/>
+      <c r="H43" s="36"/>
+      <c r="I43" s="36"/>
+      <c r="J43" s="36"/>
       <c r="K43" s="15"/>
-      <c r="L43" s="27"/>
-      <c r="M43" s="27"/>
-      <c r="N43" s="27"/>
-      <c r="O43" s="27"/>
-      <c r="P43" s="27"/>
-      <c r="Q43" s="22"/>
+      <c r="L43" s="33"/>
+      <c r="M43" s="33"/>
+      <c r="N43" s="33"/>
+      <c r="O43" s="33"/>
+      <c r="P43" s="33"/>
+      <c r="Q43" s="29"/>
     </row>
     <row r="44" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="22"/>
-      <c r="B44" s="22"/>
+      <c r="A44" s="29"/>
+      <c r="B44" s="29"/>
       <c r="C44" s="6" t="s">
         <v>46</v>
       </c>
@@ -2409,11 +2409,11 @@
       <c r="N44" s="5"/>
       <c r="O44" s="5"/>
       <c r="P44" s="5"/>
-      <c r="Q44" s="22"/>
+      <c r="Q44" s="29"/>
     </row>
     <row r="45" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A45" s="22"/>
-      <c r="B45" s="22"/>
+      <c r="A45" s="29"/>
+      <c r="B45" s="29"/>
       <c r="C45" s="6" t="s">
         <v>47</v>
       </c>
@@ -2421,11 +2421,11 @@
       <c r="E45" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="Q45" s="22"/>
+      <c r="Q45" s="29"/>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A46" s="22"/>
-      <c r="B46" s="22"/>
+      <c r="A46" s="29"/>
+      <c r="B46" s="29"/>
       <c r="C46" s="8" t="s">
         <v>33</v>
       </c>
@@ -2442,11 +2442,11 @@
       <c r="N46" s="9"/>
       <c r="O46" s="9"/>
       <c r="P46" s="9"/>
-      <c r="Q46" s="22"/>
+      <c r="Q46" s="29"/>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A47" s="22"/>
-      <c r="B47" s="22"/>
+      <c r="A47" s="29"/>
+      <c r="B47" s="29"/>
       <c r="C47" s="9"/>
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
@@ -2461,11 +2461,11 @@
       <c r="N47" s="9"/>
       <c r="O47" s="9"/>
       <c r="P47" s="9"/>
-      <c r="Q47" s="22"/>
+      <c r="Q47" s="29"/>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A48" s="22"/>
-      <c r="B48" s="22"/>
+      <c r="A48" s="29"/>
+      <c r="B48" s="29"/>
       <c r="E48" s="9"/>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -2478,11 +2478,11 @@
       <c r="N48" s="9"/>
       <c r="O48" s="9"/>
       <c r="P48" s="9"/>
-      <c r="Q48" s="22"/>
+      <c r="Q48" s="29"/>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A49" s="22"/>
-      <c r="B49" s="22"/>
+      <c r="A49" s="29"/>
+      <c r="B49" s="29"/>
       <c r="C49" s="9"/>
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
@@ -2497,11 +2497,11 @@
       <c r="N49" s="9"/>
       <c r="O49" s="9"/>
       <c r="P49" s="9"/>
-      <c r="Q49" s="22"/>
+      <c r="Q49" s="29"/>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A50" s="22"/>
-      <c r="B50" s="22"/>
+      <c r="A50" s="29"/>
+      <c r="B50" s="29"/>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
@@ -2516,11 +2516,11 @@
       <c r="N50" s="9"/>
       <c r="O50" s="9"/>
       <c r="P50" s="9"/>
-      <c r="Q50" s="22"/>
+      <c r="Q50" s="29"/>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A51" s="22"/>
-      <c r="B51" s="22"/>
+      <c r="A51" s="29"/>
+      <c r="B51" s="29"/>
       <c r="C51" s="9"/>
       <c r="D51" s="9"/>
       <c r="E51" s="9"/>
@@ -2535,11 +2535,11 @@
       <c r="N51" s="9"/>
       <c r="O51" s="9"/>
       <c r="P51" s="9"/>
-      <c r="Q51" s="22"/>
+      <c r="Q51" s="29"/>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A52" s="22"/>
-      <c r="B52" s="22"/>
+      <c r="A52" s="29"/>
+      <c r="B52" s="29"/>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
       <c r="E52" s="9"/>
@@ -2554,11 +2554,11 @@
       <c r="N52" s="9"/>
       <c r="O52" s="9"/>
       <c r="P52" s="9"/>
-      <c r="Q52" s="22"/>
+      <c r="Q52" s="29"/>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A53" s="22"/>
-      <c r="B53" s="22"/>
+      <c r="A53" s="29"/>
+      <c r="B53" s="29"/>
       <c r="C53" s="9"/>
       <c r="D53" s="9"/>
       <c r="E53" s="9"/>
@@ -2573,11 +2573,11 @@
       <c r="N53" s="9"/>
       <c r="O53" s="9"/>
       <c r="P53" s="9"/>
-      <c r="Q53" s="22"/>
+      <c r="Q53" s="29"/>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A54" s="22"/>
-      <c r="B54" s="22"/>
+      <c r="A54" s="29"/>
+      <c r="B54" s="29"/>
       <c r="C54" s="9"/>
       <c r="D54" s="9"/>
       <c r="E54" s="9"/>
@@ -2592,11 +2592,11 @@
       <c r="N54" s="9"/>
       <c r="O54" s="9"/>
       <c r="P54" s="9"/>
-      <c r="Q54" s="22"/>
+      <c r="Q54" s="29"/>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A55" s="22"/>
-      <c r="B55" s="22"/>
+      <c r="A55" s="29"/>
+      <c r="B55" s="29"/>
       <c r="C55" s="9"/>
       <c r="D55" s="9"/>
       <c r="E55" s="9"/>
@@ -2611,11 +2611,11 @@
       <c r="N55" s="9"/>
       <c r="O55" s="9"/>
       <c r="P55" s="9"/>
-      <c r="Q55" s="22"/>
+      <c r="Q55" s="29"/>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A56" s="22"/>
-      <c r="B56" s="22"/>
+      <c r="A56" s="29"/>
+      <c r="B56" s="29"/>
       <c r="C56" s="9"/>
       <c r="D56" s="9"/>
       <c r="E56" s="9"/>
@@ -2630,11 +2630,11 @@
       <c r="N56" s="9"/>
       <c r="O56" s="9"/>
       <c r="P56" s="9"/>
-      <c r="Q56" s="22"/>
+      <c r="Q56" s="29"/>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A57" s="22"/>
-      <c r="B57" s="22"/>
+      <c r="A57" s="29"/>
+      <c r="B57" s="29"/>
       <c r="C57" s="9"/>
       <c r="D57" s="9"/>
       <c r="E57" s="9"/>
@@ -2649,11 +2649,11 @@
       <c r="N57" s="9"/>
       <c r="O57" s="9"/>
       <c r="P57" s="9"/>
-      <c r="Q57" s="22"/>
+      <c r="Q57" s="29"/>
     </row>
     <row r="58" spans="1:17" ht="8.4499999999999993" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="22"/>
-      <c r="B58" s="22"/>
+      <c r="A58" s="29"/>
+      <c r="B58" s="29"/>
       <c r="C58" s="9"/>
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
@@ -2668,136 +2668,153 @@
       <c r="N58" s="9"/>
       <c r="O58" s="9"/>
       <c r="P58" s="9"/>
-      <c r="Q58" s="22"/>
+      <c r="Q58" s="29"/>
     </row>
     <row r="59" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="22"/>
-      <c r="B59" s="22"/>
-      <c r="C59" s="28" t="s">
+      <c r="A59" s="29"/>
+      <c r="B59" s="29"/>
+      <c r="C59" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="D59" s="28"/>
-      <c r="E59" s="28"/>
-      <c r="F59" s="28"/>
-      <c r="G59" s="28"/>
-      <c r="H59" s="22"/>
-      <c r="I59" s="22"/>
-      <c r="J59" s="22"/>
-      <c r="K59" s="22"/>
-      <c r="L59" s="22"/>
-      <c r="M59" s="22"/>
-      <c r="N59" s="22"/>
-      <c r="O59" s="22"/>
-      <c r="P59" s="22"/>
-      <c r="Q59" s="22"/>
+      <c r="D59" s="34"/>
+      <c r="E59" s="34"/>
+      <c r="F59" s="34"/>
+      <c r="G59" s="34"/>
+      <c r="H59" s="29"/>
+      <c r="I59" s="29"/>
+      <c r="J59" s="29"/>
+      <c r="K59" s="29"/>
+      <c r="L59" s="29"/>
+      <c r="M59" s="29"/>
+      <c r="N59" s="29"/>
+      <c r="O59" s="29"/>
+      <c r="P59" s="29"/>
+      <c r="Q59" s="29"/>
     </row>
     <row r="60" spans="1:17" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="22"/>
-      <c r="B60" s="22"/>
-      <c r="C60" s="22"/>
-      <c r="D60" s="22"/>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="22"/>
-      <c r="H60" s="22"/>
-      <c r="I60" s="22"/>
-      <c r="J60" s="22"/>
-      <c r="K60" s="22"/>
-      <c r="L60" s="22"/>
-      <c r="M60" s="22"/>
-      <c r="N60" s="22"/>
-      <c r="O60" s="22"/>
-      <c r="P60" s="22"/>
-      <c r="Q60" s="22"/>
+      <c r="A60" s="29"/>
+      <c r="B60" s="29"/>
+      <c r="C60" s="29"/>
+      <c r="D60" s="29"/>
+      <c r="E60" s="29"/>
+      <c r="F60" s="29"/>
+      <c r="G60" s="29"/>
+      <c r="H60" s="29"/>
+      <c r="I60" s="29"/>
+      <c r="J60" s="29"/>
+      <c r="K60" s="29"/>
+      <c r="L60" s="29"/>
+      <c r="M60" s="29"/>
+      <c r="N60" s="29"/>
+      <c r="O60" s="29"/>
+      <c r="P60" s="29"/>
+      <c r="Q60" s="29"/>
     </row>
     <row r="61" spans="1:17" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="22"/>
-      <c r="B61" s="22"/>
-      <c r="C61" s="22"/>
-      <c r="D61" s="22"/>
-      <c r="E61" s="22"/>
-      <c r="F61" s="22"/>
-      <c r="G61" s="22"/>
-      <c r="H61" s="22"/>
-      <c r="I61" s="22"/>
-      <c r="J61" s="22"/>
-      <c r="K61" s="22"/>
-      <c r="L61" s="22"/>
-      <c r="M61" s="22"/>
-      <c r="N61" s="22"/>
-      <c r="O61" s="22"/>
-      <c r="P61" s="22"/>
-      <c r="Q61" s="22"/>
+      <c r="A61" s="29"/>
+      <c r="B61" s="29"/>
+      <c r="C61" s="29"/>
+      <c r="D61" s="29"/>
+      <c r="E61" s="29"/>
+      <c r="F61" s="29"/>
+      <c r="G61" s="29"/>
+      <c r="H61" s="29"/>
+      <c r="I61" s="29"/>
+      <c r="J61" s="29"/>
+      <c r="K61" s="29"/>
+      <c r="L61" s="29"/>
+      <c r="M61" s="29"/>
+      <c r="N61" s="29"/>
+      <c r="O61" s="29"/>
+      <c r="P61" s="29"/>
+      <c r="Q61" s="29"/>
     </row>
     <row r="62" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A62" s="22"/>
-      <c r="B62" s="22"/>
+      <c r="A62" s="29"/>
+      <c r="B62" s="29"/>
       <c r="C62" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D62" s="38"/>
-      <c r="E62" s="39"/>
-      <c r="G62" s="22"/>
-      <c r="H62" s="22"/>
-      <c r="I62" s="22"/>
-      <c r="J62" s="22"/>
-      <c r="K62" s="22"/>
-      <c r="L62" s="22"/>
-      <c r="M62" s="22"/>
-      <c r="N62" s="26" t="s">
+      <c r="D62" s="23"/>
+      <c r="E62" s="24"/>
+      <c r="G62" s="29"/>
+      <c r="H62" s="29"/>
+      <c r="I62" s="29"/>
+      <c r="J62" s="29"/>
+      <c r="K62" s="29"/>
+      <c r="L62" s="29"/>
+      <c r="M62" s="29"/>
+      <c r="N62" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="O62" s="26"/>
-      <c r="P62" s="26"/>
-      <c r="Q62" s="22"/>
+      <c r="O62" s="32"/>
+      <c r="P62" s="32"/>
+      <c r="Q62" s="29"/>
     </row>
     <row r="63" spans="1:17" ht="13.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="22"/>
-      <c r="B63" s="22"/>
-      <c r="C63" s="22"/>
-      <c r="D63" s="22"/>
-      <c r="E63" s="22"/>
-      <c r="F63" s="22"/>
-      <c r="G63" s="22"/>
-      <c r="H63" s="22"/>
-      <c r="I63" s="22"/>
-      <c r="J63" s="22"/>
-      <c r="K63" s="22"/>
-      <c r="L63" s="22"/>
-      <c r="M63" s="22"/>
-      <c r="N63" s="22"/>
-      <c r="O63" s="22"/>
-      <c r="P63" s="22"/>
-      <c r="Q63" s="22"/>
+      <c r="A63" s="29"/>
+      <c r="B63" s="29"/>
+      <c r="C63" s="29"/>
+      <c r="D63" s="29"/>
+      <c r="E63" s="29"/>
+      <c r="F63" s="29"/>
+      <c r="G63" s="29"/>
+      <c r="H63" s="29"/>
+      <c r="I63" s="29"/>
+      <c r="J63" s="29"/>
+      <c r="K63" s="29"/>
+      <c r="L63" s="29"/>
+      <c r="M63" s="29"/>
+      <c r="N63" s="29"/>
+      <c r="O63" s="29"/>
+      <c r="P63" s="29"/>
+      <c r="Q63" s="29"/>
     </row>
     <row r="64" spans="1:17" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="22"/>
-      <c r="C64" s="22"/>
-      <c r="D64" s="22"/>
-      <c r="E64" s="22"/>
-      <c r="F64" s="22"/>
-      <c r="G64" s="22"/>
-      <c r="H64" s="22"/>
-      <c r="I64" s="22"/>
-      <c r="J64" s="22"/>
-      <c r="K64" s="22"/>
-      <c r="L64" s="22"/>
-      <c r="M64" s="22"/>
-      <c r="N64" s="22"/>
-      <c r="O64" s="22"/>
-      <c r="P64" s="22"/>
-      <c r="Q64" s="22"/>
+      <c r="B64" s="29"/>
+      <c r="C64" s="29"/>
+      <c r="D64" s="29"/>
+      <c r="E64" s="29"/>
+      <c r="F64" s="29"/>
+      <c r="G64" s="29"/>
+      <c r="H64" s="29"/>
+      <c r="I64" s="29"/>
+      <c r="J64" s="29"/>
+      <c r="K64" s="29"/>
+      <c r="L64" s="29"/>
+      <c r="M64" s="29"/>
+      <c r="N64" s="29"/>
+      <c r="O64" s="29"/>
+      <c r="P64" s="29"/>
+      <c r="Q64" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="F6:J6"/>
-    <mergeCell ref="F7:J7"/>
-    <mergeCell ref="F14:J14"/>
-    <mergeCell ref="F22:J22"/>
-    <mergeCell ref="F35:J35"/>
-    <mergeCell ref="C15:P16"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C42:P42"/>
+    <mergeCell ref="L29:P31"/>
+    <mergeCell ref="C23:P23"/>
+    <mergeCell ref="C25:P25"/>
+    <mergeCell ref="L35:P37"/>
+    <mergeCell ref="C34:P34"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="L26:O26"/>
+    <mergeCell ref="B63:Q64"/>
+    <mergeCell ref="C38:P38"/>
+    <mergeCell ref="N62:P62"/>
+    <mergeCell ref="L43:P43"/>
+    <mergeCell ref="C59:G59"/>
+    <mergeCell ref="B2:B62"/>
+    <mergeCell ref="F9:J9"/>
+    <mergeCell ref="F12:J12"/>
+    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="F8:J8"/>
+    <mergeCell ref="H21:N21"/>
+    <mergeCell ref="F28:J28"/>
+    <mergeCell ref="F30:J30"/>
+    <mergeCell ref="H41:M41"/>
+    <mergeCell ref="C5:P5"/>
+    <mergeCell ref="F43:J43"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="Q2:Q62"/>
     <mergeCell ref="L22:P22"/>
@@ -2814,31 +2831,14 @@
     <mergeCell ref="C18:P18"/>
     <mergeCell ref="G62:M62"/>
     <mergeCell ref="A2:A63"/>
-    <mergeCell ref="B63:Q64"/>
-    <mergeCell ref="C38:P38"/>
-    <mergeCell ref="N62:P62"/>
-    <mergeCell ref="L43:P43"/>
-    <mergeCell ref="C59:G59"/>
-    <mergeCell ref="B2:B62"/>
-    <mergeCell ref="F9:J9"/>
-    <mergeCell ref="F12:J12"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="F8:J8"/>
-    <mergeCell ref="H21:N21"/>
-    <mergeCell ref="F28:J28"/>
-    <mergeCell ref="F30:J30"/>
-    <mergeCell ref="H41:M41"/>
-    <mergeCell ref="C5:P5"/>
-    <mergeCell ref="F43:J43"/>
-    <mergeCell ref="C42:P42"/>
-    <mergeCell ref="L29:P31"/>
-    <mergeCell ref="C23:P23"/>
-    <mergeCell ref="C25:P25"/>
-    <mergeCell ref="L35:P37"/>
-    <mergeCell ref="C34:P34"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="L26:O26"/>
+    <mergeCell ref="F6:J6"/>
+    <mergeCell ref="F7:J7"/>
+    <mergeCell ref="F14:J14"/>
+    <mergeCell ref="F22:J22"/>
+    <mergeCell ref="F35:J35"/>
+    <mergeCell ref="C15:P16"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C22:D22"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="81" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
created a modification for the excecl template, modifued using open pyxel then transfer to pdf
</commit_message>
<xml_diff>
--- a/core/main/templates/print_excel/cmf_template.xlsx
+++ b/core/main/templates/print_excel/cmf_template.xlsx
@@ -397,46 +397,46 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1461,105 +1461,105 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="29"/>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
+      <c r="A1" s="25"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="29"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-      <c r="P2" s="29"/>
-      <c r="Q2" s="29"/>
+      <c r="A2" s="25"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="25"/>
+      <c r="P2" s="25"/>
+      <c r="Q2" s="25"/>
     </row>
     <row r="3" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="29"/>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="31" t="s">
+      <c r="A3" s="25"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="N3" s="31"/>
-      <c r="O3" s="31"/>
-      <c r="P3" s="31"/>
-      <c r="Q3" s="29"/>
+      <c r="N3" s="36"/>
+      <c r="O3" s="36"/>
+      <c r="P3" s="36"/>
+      <c r="Q3" s="25"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="29"/>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29"/>
-      <c r="K4" s="29"/>
-      <c r="L4" s="29"/>
-      <c r="M4" s="29"/>
-      <c r="N4" s="29"/>
-      <c r="O4" s="29"/>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="29"/>
+      <c r="A4" s="25"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="25"/>
+      <c r="N4" s="25"/>
+      <c r="O4" s="25"/>
+      <c r="P4" s="25"/>
+      <c r="Q4" s="25"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="29"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="29"/>
-      <c r="K5" s="29"/>
-      <c r="L5" s="29"/>
-      <c r="M5" s="29"/>
-      <c r="N5" s="29"/>
-      <c r="O5" s="29"/>
-      <c r="P5" s="29"/>
-      <c r="Q5" s="29"/>
+      <c r="A5" s="25"/>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="25"/>
+      <c r="J5" s="25"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="25"/>
+      <c r="N5" s="25"/>
+      <c r="O5" s="25"/>
+      <c r="P5" s="25"/>
+      <c r="Q5" s="25"/>
     </row>
     <row r="6" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="29"/>
-      <c r="B6" s="29"/>
+      <c r="A6" s="25"/>
+      <c r="B6" s="25"/>
       <c r="C6" s="1" t="s">
         <v>35</v>
       </c>
@@ -1567,22 +1567,22 @@
       <c r="E6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="25"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28"/>
       <c r="K6" s="1"/>
-      <c r="L6" s="29"/>
-      <c r="M6" s="29"/>
-      <c r="N6" s="29"/>
-      <c r="O6" s="29"/>
-      <c r="P6" s="29"/>
-      <c r="Q6" s="29"/>
+      <c r="L6" s="25"/>
+      <c r="M6" s="25"/>
+      <c r="N6" s="25"/>
+      <c r="O6" s="25"/>
+      <c r="P6" s="25"/>
+      <c r="Q6" s="25"/>
     </row>
     <row r="7" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="29"/>
-      <c r="B7" s="29"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="25"/>
       <c r="C7" s="6" t="s">
         <v>1</v>
       </c>
@@ -1590,22 +1590,22 @@
       <c r="E7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="26"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
       <c r="K7" s="13"/>
       <c r="L7" s="10"/>
       <c r="M7" s="10"/>
       <c r="N7" s="10"/>
       <c r="O7" s="10"/>
       <c r="P7" s="1"/>
-      <c r="Q7" s="29"/>
+      <c r="Q7" s="25"/>
     </row>
     <row r="8" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="29"/>
-      <c r="B8" s="29"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="25"/>
       <c r="C8" s="6" t="s">
         <v>2</v>
       </c>
@@ -1613,17 +1613,17 @@
       <c r="E8" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="35"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="32"/>
       <c r="K8" s="17"/>
-      <c r="Q8" s="29"/>
+      <c r="Q8" s="25"/>
     </row>
     <row r="9" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="29"/>
-      <c r="B9" s="29"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="25"/>
       <c r="C9" s="6" t="s">
         <v>40</v>
       </c>
@@ -1631,31 +1631,31 @@
       <c r="E9" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="32"/>
       <c r="K9" s="17"/>
-      <c r="Q9" s="29"/>
+      <c r="Q9" s="25"/>
     </row>
     <row r="10" spans="1:17" ht="3.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="29"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
+      <c r="A10" s="25"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="25"/>
       <c r="K10" s="12"/>
-      <c r="Q10" s="29"/>
+      <c r="Q10" s="25"/>
     </row>
     <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="29"/>
-      <c r="B11" s="29"/>
+      <c r="A11" s="25"/>
+      <c r="B11" s="25"/>
       <c r="C11" s="6" t="s">
         <v>3</v>
       </c>
@@ -1674,11 +1674,11 @@
         <v>9</v>
       </c>
       <c r="K11" s="1"/>
-      <c r="Q11" s="29"/>
+      <c r="Q11" s="25"/>
     </row>
     <row r="12" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="29"/>
-      <c r="B12" s="29"/>
+      <c r="A12" s="25"/>
+      <c r="B12" s="25"/>
       <c r="C12" s="6" t="s">
         <v>5</v>
       </c>
@@ -1686,22 +1686,22 @@
       <c r="E12" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="36"/>
-      <c r="I12" s="36"/>
-      <c r="J12" s="36"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="13"/>
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
       <c r="O12" s="10"/>
       <c r="P12" s="1"/>
-      <c r="Q12" s="29"/>
+      <c r="Q12" s="25"/>
     </row>
     <row r="13" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="29"/>
-      <c r="B13" s="29"/>
+      <c r="A13" s="25"/>
+      <c r="B13" s="25"/>
       <c r="C13" s="6" t="s">
         <v>6</v>
       </c>
@@ -1709,22 +1709,22 @@
       <c r="E13" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="26"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="34"/>
+      <c r="J13" s="34"/>
       <c r="K13" s="14"/>
       <c r="L13" s="11"/>
       <c r="M13" s="11"/>
       <c r="N13" s="11"/>
       <c r="O13" s="11"/>
       <c r="P13" s="1"/>
-      <c r="Q13" s="29"/>
+      <c r="Q13" s="25"/>
     </row>
     <row r="14" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="29"/>
-      <c r="B14" s="29"/>
+      <c r="A14" s="25"/>
+      <c r="B14" s="25"/>
       <c r="C14" s="6" t="s">
         <v>7</v>
       </c>
@@ -1732,60 +1732,60 @@
       <c r="E14" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
+      <c r="F14" s="37"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="37"/>
+      <c r="J14" s="37"/>
       <c r="K14" s="10"/>
       <c r="L14" s="10"/>
       <c r="M14" s="10"/>
       <c r="N14" s="10"/>
       <c r="O14" s="10"/>
       <c r="P14" s="1"/>
-      <c r="Q14" s="29"/>
+      <c r="Q14" s="25"/>
     </row>
     <row r="15" spans="1:17" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="29"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="29"/>
-      <c r="H15" s="29"/>
-      <c r="I15" s="29"/>
-      <c r="J15" s="29"/>
-      <c r="K15" s="29"/>
-      <c r="L15" s="29"/>
-      <c r="M15" s="29"/>
-      <c r="N15" s="29"/>
-      <c r="O15" s="29"/>
-      <c r="P15" s="29"/>
-      <c r="Q15" s="29"/>
+      <c r="A15" s="25"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="25"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="25"/>
+      <c r="M15" s="25"/>
+      <c r="N15" s="25"/>
+      <c r="O15" s="25"/>
+      <c r="P15" s="25"/>
+      <c r="Q15" s="25"/>
     </row>
     <row r="16" spans="1:17" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="29"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="29"/>
-      <c r="H16" s="29"/>
-      <c r="I16" s="29"/>
-      <c r="J16" s="29"/>
-      <c r="K16" s="29"/>
-      <c r="L16" s="29"/>
-      <c r="M16" s="29"/>
-      <c r="N16" s="29"/>
-      <c r="O16" s="29"/>
-      <c r="P16" s="29"/>
-      <c r="Q16" s="29"/>
+      <c r="A16" s="25"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="25"/>
+      <c r="M16" s="25"/>
+      <c r="N16" s="25"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="25"/>
+      <c r="Q16" s="25"/>
     </row>
     <row r="17" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="29"/>
-      <c r="B17" s="29"/>
+      <c r="A17" s="25"/>
+      <c r="B17" s="25"/>
       <c r="C17" s="6" t="s">
         <v>41</v>
       </c>
@@ -1812,30 +1812,30 @@
       <c r="M17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="Q17" s="29"/>
+      <c r="Q17" s="25"/>
     </row>
     <row r="18" spans="1:17" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="29"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="29"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="29"/>
-      <c r="J18" s="29"/>
-      <c r="K18" s="29"/>
-      <c r="L18" s="29"/>
-      <c r="M18" s="29"/>
-      <c r="N18" s="29"/>
-      <c r="O18" s="29"/>
-      <c r="P18" s="29"/>
-      <c r="Q18" s="29"/>
+      <c r="A18" s="25"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="25"/>
+      <c r="L18" s="25"/>
+      <c r="M18" s="25"/>
+      <c r="N18" s="25"/>
+      <c r="O18" s="25"/>
+      <c r="P18" s="25"/>
+      <c r="Q18" s="25"/>
     </row>
     <row r="19" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="29"/>
-      <c r="B19" s="29"/>
+      <c r="A19" s="25"/>
+      <c r="B19" s="25"/>
       <c r="F19" s="16" t="b">
         <v>0</v>
       </c>
@@ -1855,84 +1855,84 @@
       <c r="M19" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q19" s="29"/>
+      <c r="Q19" s="25"/>
     </row>
     <row r="20" spans="1:17" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="29"/>
-      <c r="B20" s="29"/>
+      <c r="A20" s="25"/>
+      <c r="B20" s="25"/>
       <c r="G20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
       <c r="M20" s="1"/>
-      <c r="Q20" s="29"/>
+      <c r="Q20" s="25"/>
     </row>
     <row r="21" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="29"/>
-      <c r="B21" s="29"/>
+      <c r="A21" s="25"/>
+      <c r="B21" s="25"/>
       <c r="F21" s="22" t="b">
         <v>0</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H21" s="37"/>
-      <c r="I21" s="37"/>
-      <c r="J21" s="37"/>
-      <c r="K21" s="37"/>
-      <c r="L21" s="37"/>
-      <c r="M21" s="37"/>
-      <c r="N21" s="37"/>
-      <c r="Q21" s="29"/>
+      <c r="H21" s="35"/>
+      <c r="I21" s="35"/>
+      <c r="J21" s="35"/>
+      <c r="K21" s="35"/>
+      <c r="L21" s="35"/>
+      <c r="M21" s="35"/>
+      <c r="N21" s="35"/>
+      <c r="Q21" s="25"/>
     </row>
     <row r="22" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="30" t="s">
+      <c r="A22" s="25"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="30"/>
+      <c r="D22" s="39"/>
       <c r="E22" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="25"/>
-      <c r="J22" s="25"/>
+      <c r="F22" s="28"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="28"/>
+      <c r="J22" s="28"/>
       <c r="K22" s="1"/>
-      <c r="L22" s="29"/>
-      <c r="M22" s="29"/>
-      <c r="N22" s="29"/>
-      <c r="O22" s="29"/>
-      <c r="P22" s="29"/>
-      <c r="Q22" s="29"/>
+      <c r="L22" s="25"/>
+      <c r="M22" s="25"/>
+      <c r="N22" s="25"/>
+      <c r="O22" s="25"/>
+      <c r="P22" s="25"/>
+      <c r="Q22" s="25"/>
     </row>
     <row r="23" spans="1:17" ht="4.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="29"/>
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="29"/>
-      <c r="I23" s="29"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="29"/>
-      <c r="L23" s="29"/>
-      <c r="M23" s="29"/>
-      <c r="N23" s="29"/>
-      <c r="O23" s="29"/>
-      <c r="P23" s="29"/>
-      <c r="Q23" s="29"/>
+      <c r="A23" s="25"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="25"/>
+      <c r="K23" s="25"/>
+      <c r="L23" s="25"/>
+      <c r="M23" s="25"/>
+      <c r="N23" s="25"/>
+      <c r="O23" s="25"/>
+      <c r="P23" s="25"/>
+      <c r="Q23" s="25"/>
     </row>
     <row r="24" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="29"/>
-      <c r="B24" s="29"/>
-      <c r="C24" s="30" t="s">
+      <c r="A24" s="25"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="D24" s="30"/>
+      <c r="D24" s="39"/>
       <c r="E24" s="2" t="s">
         <v>4</v>
       </c>
@@ -1955,32 +1955,32 @@
       <c r="N24" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="O24" s="29"/>
-      <c r="P24" s="29"/>
-      <c r="Q24" s="29"/>
+      <c r="O24" s="25"/>
+      <c r="P24" s="25"/>
+      <c r="Q24" s="25"/>
     </row>
     <row r="25" spans="1:17" ht="4.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="29"/>
-      <c r="B25" s="29"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="29"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="29"/>
-      <c r="K25" s="29"/>
-      <c r="L25" s="29"/>
-      <c r="M25" s="29"/>
-      <c r="N25" s="29"/>
-      <c r="O25" s="29"/>
-      <c r="P25" s="29"/>
-      <c r="Q25" s="29"/>
+      <c r="A25" s="25"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="25"/>
+      <c r="I25" s="25"/>
+      <c r="J25" s="25"/>
+      <c r="K25" s="25"/>
+      <c r="L25" s="25"/>
+      <c r="M25" s="25"/>
+      <c r="N25" s="25"/>
+      <c r="O25" s="25"/>
+      <c r="P25" s="25"/>
+      <c r="Q25" s="25"/>
     </row>
     <row r="26" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="29"/>
-      <c r="B26" s="29"/>
+      <c r="A26" s="25"/>
+      <c r="B26" s="25"/>
       <c r="F26" s="21" t="b">
         <v>0</v>
       </c>
@@ -1994,31 +1994,31 @@
         <v>38</v>
       </c>
       <c r="K26" s="1"/>
-      <c r="L26" s="25"/>
-      <c r="M26" s="25"/>
-      <c r="N26" s="25"/>
-      <c r="O26" s="25"/>
-      <c r="Q26" s="29"/>
+      <c r="L26" s="28"/>
+      <c r="M26" s="28"/>
+      <c r="N26" s="28"/>
+      <c r="O26" s="28"/>
+      <c r="Q26" s="25"/>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A27" s="29"/>
-      <c r="B27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="29"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="29"/>
-      <c r="K27" s="29"/>
-      <c r="L27" s="29"/>
-      <c r="M27" s="29"/>
-      <c r="N27" s="29"/>
-      <c r="O27" s="29"/>
-      <c r="P27" s="29"/>
-      <c r="Q27" s="29"/>
+      <c r="A27" s="25"/>
+      <c r="B27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="25"/>
+      <c r="K27" s="25"/>
+      <c r="L27" s="25"/>
+      <c r="M27" s="25"/>
+      <c r="N27" s="25"/>
+      <c r="O27" s="25"/>
+      <c r="P27" s="25"/>
+      <c r="Q27" s="25"/>
     </row>
     <row r="28" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="29"/>
-      <c r="B28" s="29"/>
+      <c r="A28" s="25"/>
+      <c r="B28" s="25"/>
       <c r="C28" s="6" t="s">
         <v>20</v>
       </c>
@@ -2026,22 +2026,22 @@
       <c r="E28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F28" s="36"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="36"/>
-      <c r="I28" s="36"/>
-      <c r="J28" s="36"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="15"/>
       <c r="L28" s="3"/>
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
-      <c r="Q28" s="29"/>
+      <c r="Q28" s="25"/>
     </row>
     <row r="29" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="29"/>
-      <c r="B29" s="29"/>
+      <c r="A29" s="25"/>
+      <c r="B29" s="25"/>
       <c r="C29" s="6" t="s">
         <v>44</v>
       </c>
@@ -2062,18 +2062,18 @@
         <v>22</v>
       </c>
       <c r="K29" s="1"/>
-      <c r="L29" s="38" t="s">
+      <c r="L29" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="M29" s="38"/>
-      <c r="N29" s="38"/>
-      <c r="O29" s="38"/>
-      <c r="P29" s="38"/>
-      <c r="Q29" s="29"/>
+      <c r="M29" s="26"/>
+      <c r="N29" s="26"/>
+      <c r="O29" s="26"/>
+      <c r="P29" s="26"/>
+      <c r="Q29" s="25"/>
     </row>
     <row r="30" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="29"/>
-      <c r="B30" s="29"/>
+      <c r="A30" s="25"/>
+      <c r="B30" s="25"/>
       <c r="C30" s="6" t="s">
         <v>45</v>
       </c>
@@ -2081,22 +2081,22 @@
       <c r="E30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F30" s="36"/>
-      <c r="G30" s="36"/>
-      <c r="H30" s="36"/>
-      <c r="I30" s="36"/>
-      <c r="J30" s="36"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="33"/>
       <c r="K30" s="15"/>
-      <c r="L30" s="38"/>
-      <c r="M30" s="38"/>
-      <c r="N30" s="38"/>
-      <c r="O30" s="38"/>
-      <c r="P30" s="38"/>
-      <c r="Q30" s="29"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
+      <c r="N30" s="26"/>
+      <c r="O30" s="26"/>
+      <c r="P30" s="26"/>
+      <c r="Q30" s="25"/>
     </row>
     <row r="31" spans="1:17" ht="21.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="29"/>
-      <c r="B31" s="29"/>
+      <c r="A31" s="25"/>
+      <c r="B31" s="25"/>
       <c r="C31" s="1" t="s">
         <v>31</v>
       </c>
@@ -2117,35 +2117,35 @@
         <v>22</v>
       </c>
       <c r="K31" s="1"/>
-      <c r="L31" s="38"/>
-      <c r="M31" s="38"/>
-      <c r="N31" s="38"/>
-      <c r="O31" s="38"/>
-      <c r="P31" s="38"/>
-      <c r="Q31" s="29"/>
+      <c r="L31" s="26"/>
+      <c r="M31" s="26"/>
+      <c r="N31" s="26"/>
+      <c r="O31" s="26"/>
+      <c r="P31" s="26"/>
+      <c r="Q31" s="25"/>
     </row>
     <row r="32" spans="1:17" ht="4.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="29"/>
-      <c r="B32" s="29"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="29"/>
-      <c r="J32" s="29"/>
-      <c r="K32" s="29"/>
-      <c r="L32" s="29"/>
-      <c r="M32" s="29"/>
-      <c r="N32" s="29"/>
-      <c r="O32" s="29"/>
-      <c r="P32" s="29"/>
-      <c r="Q32" s="29"/>
+      <c r="A32" s="25"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="25"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="25"/>
+      <c r="K32" s="25"/>
+      <c r="L32" s="25"/>
+      <c r="M32" s="25"/>
+      <c r="N32" s="25"/>
+      <c r="O32" s="25"/>
+      <c r="P32" s="25"/>
+      <c r="Q32" s="25"/>
     </row>
     <row r="33" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="29"/>
-      <c r="B33" s="29"/>
+      <c r="A33" s="25"/>
+      <c r="B33" s="25"/>
       <c r="C33" s="6" t="s">
         <v>23</v>
       </c>
@@ -2172,32 +2172,32 @@
       <c r="M33" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="O33" s="25"/>
-      <c r="P33" s="25"/>
-      <c r="Q33" s="29"/>
+      <c r="O33" s="28"/>
+      <c r="P33" s="28"/>
+      <c r="Q33" s="25"/>
     </row>
     <row r="34" spans="1:17" ht="4.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="29"/>
-      <c r="B34" s="29"/>
-      <c r="C34" s="29"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="29"/>
-      <c r="F34" s="29"/>
-      <c r="G34" s="29"/>
-      <c r="H34" s="29"/>
-      <c r="I34" s="29"/>
-      <c r="J34" s="29"/>
-      <c r="K34" s="29"/>
-      <c r="L34" s="29"/>
-      <c r="M34" s="29"/>
-      <c r="N34" s="29"/>
-      <c r="O34" s="29"/>
-      <c r="P34" s="29"/>
-      <c r="Q34" s="29"/>
+      <c r="A34" s="25"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="25"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="25"/>
+      <c r="K34" s="25"/>
+      <c r="L34" s="25"/>
+      <c r="M34" s="25"/>
+      <c r="N34" s="25"/>
+      <c r="O34" s="25"/>
+      <c r="P34" s="25"/>
+      <c r="Q34" s="25"/>
     </row>
     <row r="35" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="29"/>
-      <c r="B35" s="29"/>
+      <c r="A35" s="25"/>
+      <c r="B35" s="25"/>
       <c r="C35" s="7" t="s">
         <v>36</v>
       </c>
@@ -2205,32 +2205,32 @@
       <c r="E35" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F35" s="28"/>
-      <c r="G35" s="28"/>
-      <c r="H35" s="28"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="28"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="38"/>
+      <c r="J35" s="38"/>
       <c r="K35" s="18"/>
-      <c r="L35" s="39"/>
-      <c r="M35" s="39"/>
-      <c r="N35" s="39"/>
-      <c r="O35" s="39"/>
-      <c r="P35" s="39"/>
-      <c r="Q35" s="29"/>
+      <c r="L35" s="27"/>
+      <c r="M35" s="27"/>
+      <c r="N35" s="27"/>
+      <c r="O35" s="27"/>
+      <c r="P35" s="27"/>
+      <c r="Q35" s="25"/>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A36" s="29"/>
-      <c r="B36" s="29"/>
-      <c r="L36" s="39"/>
-      <c r="M36" s="39"/>
-      <c r="N36" s="39"/>
-      <c r="O36" s="39"/>
-      <c r="P36" s="39"/>
-      <c r="Q36" s="29"/>
+      <c r="A36" s="25"/>
+      <c r="B36" s="25"/>
+      <c r="L36" s="27"/>
+      <c r="M36" s="27"/>
+      <c r="N36" s="27"/>
+      <c r="O36" s="27"/>
+      <c r="P36" s="27"/>
+      <c r="Q36" s="25"/>
     </row>
     <row r="37" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="29"/>
-      <c r="B37" s="29"/>
+      <c r="A37" s="25"/>
+      <c r="B37" s="25"/>
       <c r="C37" s="1" t="s">
         <v>26</v>
       </c>
@@ -2251,35 +2251,35 @@
         <v>22</v>
       </c>
       <c r="K37" s="1"/>
-      <c r="L37" s="39"/>
-      <c r="M37" s="39"/>
-      <c r="N37" s="39"/>
-      <c r="O37" s="39"/>
-      <c r="P37" s="39"/>
-      <c r="Q37" s="29"/>
+      <c r="L37" s="27"/>
+      <c r="M37" s="27"/>
+      <c r="N37" s="27"/>
+      <c r="O37" s="27"/>
+      <c r="P37" s="27"/>
+      <c r="Q37" s="25"/>
     </row>
     <row r="38" spans="1:17" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="29"/>
-      <c r="B38" s="29"/>
-      <c r="C38" s="29"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="29"/>
-      <c r="G38" s="29"/>
-      <c r="H38" s="29"/>
-      <c r="I38" s="29"/>
-      <c r="J38" s="29"/>
-      <c r="K38" s="29"/>
-      <c r="L38" s="29"/>
-      <c r="M38" s="29"/>
-      <c r="N38" s="29"/>
-      <c r="O38" s="29"/>
-      <c r="P38" s="29"/>
-      <c r="Q38" s="29"/>
+      <c r="A38" s="25"/>
+      <c r="B38" s="25"/>
+      <c r="C38" s="25"/>
+      <c r="D38" s="25"/>
+      <c r="E38" s="25"/>
+      <c r="F38" s="25"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="25"/>
+      <c r="I38" s="25"/>
+      <c r="J38" s="25"/>
+      <c r="K38" s="25"/>
+      <c r="L38" s="25"/>
+      <c r="M38" s="25"/>
+      <c r="N38" s="25"/>
+      <c r="O38" s="25"/>
+      <c r="P38" s="25"/>
+      <c r="Q38" s="25"/>
     </row>
     <row r="39" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" s="29"/>
-      <c r="B39" s="29"/>
+      <c r="A39" s="25"/>
+      <c r="B39" s="25"/>
       <c r="C39" s="6" t="s">
         <v>27</v>
       </c>
@@ -2300,11 +2300,11 @@
         <v>29</v>
       </c>
       <c r="K39" s="1"/>
-      <c r="Q39" s="29"/>
+      <c r="Q39" s="25"/>
     </row>
     <row r="40" spans="1:17" ht="3.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="29"/>
-      <c r="B40" s="29"/>
+      <c r="A40" s="25"/>
+      <c r="B40" s="25"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
@@ -2314,11 +2314,11 @@
       <c r="K40" s="1"/>
       <c r="N40" s="1"/>
       <c r="P40" s="1"/>
-      <c r="Q40" s="29"/>
+      <c r="Q40" s="25"/>
     </row>
     <row r="41" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="29"/>
-      <c r="B41" s="29"/>
+      <c r="A41" s="25"/>
+      <c r="B41" s="25"/>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
@@ -2328,38 +2328,38 @@
       <c r="G41" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H41" s="37"/>
-      <c r="I41" s="37"/>
-      <c r="J41" s="37"/>
-      <c r="K41" s="37"/>
-      <c r="L41" s="37"/>
-      <c r="M41" s="37"/>
+      <c r="H41" s="35"/>
+      <c r="I41" s="35"/>
+      <c r="J41" s="35"/>
+      <c r="K41" s="35"/>
+      <c r="L41" s="35"/>
+      <c r="M41" s="35"/>
       <c r="N41" s="1"/>
       <c r="P41" s="1"/>
-      <c r="Q41" s="29"/>
+      <c r="Q41" s="25"/>
     </row>
     <row r="42" spans="1:17" ht="3.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="29"/>
-      <c r="B42" s="29"/>
-      <c r="C42" s="29"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="29"/>
-      <c r="H42" s="29"/>
-      <c r="I42" s="29"/>
-      <c r="J42" s="29"/>
-      <c r="K42" s="29"/>
-      <c r="L42" s="29"/>
-      <c r="M42" s="29"/>
-      <c r="N42" s="29"/>
-      <c r="O42" s="29"/>
-      <c r="P42" s="29"/>
-      <c r="Q42" s="29"/>
+      <c r="A42" s="25"/>
+      <c r="B42" s="25"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="25"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="25"/>
+      <c r="I42" s="25"/>
+      <c r="J42" s="25"/>
+      <c r="K42" s="25"/>
+      <c r="L42" s="25"/>
+      <c r="M42" s="25"/>
+      <c r="N42" s="25"/>
+      <c r="O42" s="25"/>
+      <c r="P42" s="25"/>
+      <c r="Q42" s="25"/>
     </row>
     <row r="43" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="29"/>
-      <c r="B43" s="29"/>
+      <c r="A43" s="25"/>
+      <c r="B43" s="25"/>
       <c r="C43" s="6" t="s">
         <v>30</v>
       </c>
@@ -2367,22 +2367,22 @@
       <c r="E43" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F43" s="36"/>
-      <c r="G43" s="36"/>
-      <c r="H43" s="36"/>
-      <c r="I43" s="36"/>
-      <c r="J43" s="36"/>
+      <c r="F43" s="33"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="33"/>
+      <c r="I43" s="33"/>
+      <c r="J43" s="33"/>
       <c r="K43" s="15"/>
-      <c r="L43" s="33"/>
-      <c r="M43" s="33"/>
-      <c r="N43" s="33"/>
-      <c r="O43" s="33"/>
-      <c r="P43" s="33"/>
-      <c r="Q43" s="29"/>
+      <c r="L43" s="30"/>
+      <c r="M43" s="30"/>
+      <c r="N43" s="30"/>
+      <c r="O43" s="30"/>
+      <c r="P43" s="30"/>
+      <c r="Q43" s="25"/>
     </row>
     <row r="44" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="29"/>
-      <c r="B44" s="29"/>
+      <c r="A44" s="25"/>
+      <c r="B44" s="25"/>
       <c r="C44" s="6" t="s">
         <v>46</v>
       </c>
@@ -2409,11 +2409,11 @@
       <c r="N44" s="5"/>
       <c r="O44" s="5"/>
       <c r="P44" s="5"/>
-      <c r="Q44" s="29"/>
+      <c r="Q44" s="25"/>
     </row>
     <row r="45" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A45" s="29"/>
-      <c r="B45" s="29"/>
+      <c r="A45" s="25"/>
+      <c r="B45" s="25"/>
       <c r="C45" s="6" t="s">
         <v>47</v>
       </c>
@@ -2421,11 +2421,11 @@
       <c r="E45" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="Q45" s="29"/>
+      <c r="Q45" s="25"/>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A46" s="29"/>
-      <c r="B46" s="29"/>
+      <c r="A46" s="25"/>
+      <c r="B46" s="25"/>
       <c r="C46" s="8" t="s">
         <v>33</v>
       </c>
@@ -2442,11 +2442,11 @@
       <c r="N46" s="9"/>
       <c r="O46" s="9"/>
       <c r="P46" s="9"/>
-      <c r="Q46" s="29"/>
+      <c r="Q46" s="25"/>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A47" s="29"/>
-      <c r="B47" s="29"/>
+      <c r="A47" s="25"/>
+      <c r="B47" s="25"/>
       <c r="C47" s="9"/>
       <c r="D47" s="9"/>
       <c r="E47" s="9"/>
@@ -2461,11 +2461,11 @@
       <c r="N47" s="9"/>
       <c r="O47" s="9"/>
       <c r="P47" s="9"/>
-      <c r="Q47" s="29"/>
+      <c r="Q47" s="25"/>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A48" s="29"/>
-      <c r="B48" s="29"/>
+      <c r="A48" s="25"/>
+      <c r="B48" s="25"/>
       <c r="E48" s="9"/>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -2478,11 +2478,11 @@
       <c r="N48" s="9"/>
       <c r="O48" s="9"/>
       <c r="P48" s="9"/>
-      <c r="Q48" s="29"/>
+      <c r="Q48" s="25"/>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A49" s="29"/>
-      <c r="B49" s="29"/>
+      <c r="A49" s="25"/>
+      <c r="B49" s="25"/>
       <c r="C49" s="9"/>
       <c r="D49" s="9"/>
       <c r="E49" s="9"/>
@@ -2497,11 +2497,11 @@
       <c r="N49" s="9"/>
       <c r="O49" s="9"/>
       <c r="P49" s="9"/>
-      <c r="Q49" s="29"/>
+      <c r="Q49" s="25"/>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A50" s="29"/>
-      <c r="B50" s="29"/>
+      <c r="A50" s="25"/>
+      <c r="B50" s="25"/>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
@@ -2516,11 +2516,11 @@
       <c r="N50" s="9"/>
       <c r="O50" s="9"/>
       <c r="P50" s="9"/>
-      <c r="Q50" s="29"/>
+      <c r="Q50" s="25"/>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A51" s="29"/>
-      <c r="B51" s="29"/>
+      <c r="A51" s="25"/>
+      <c r="B51" s="25"/>
       <c r="C51" s="9"/>
       <c r="D51" s="9"/>
       <c r="E51" s="9"/>
@@ -2535,11 +2535,11 @@
       <c r="N51" s="9"/>
       <c r="O51" s="9"/>
       <c r="P51" s="9"/>
-      <c r="Q51" s="29"/>
+      <c r="Q51" s="25"/>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A52" s="29"/>
-      <c r="B52" s="29"/>
+      <c r="A52" s="25"/>
+      <c r="B52" s="25"/>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
       <c r="E52" s="9"/>
@@ -2554,11 +2554,11 @@
       <c r="N52" s="9"/>
       <c r="O52" s="9"/>
       <c r="P52" s="9"/>
-      <c r="Q52" s="29"/>
+      <c r="Q52" s="25"/>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A53" s="29"/>
-      <c r="B53" s="29"/>
+      <c r="A53" s="25"/>
+      <c r="B53" s="25"/>
       <c r="C53" s="9"/>
       <c r="D53" s="9"/>
       <c r="E53" s="9"/>
@@ -2573,11 +2573,11 @@
       <c r="N53" s="9"/>
       <c r="O53" s="9"/>
       <c r="P53" s="9"/>
-      <c r="Q53" s="29"/>
+      <c r="Q53" s="25"/>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A54" s="29"/>
-      <c r="B54" s="29"/>
+      <c r="A54" s="25"/>
+      <c r="B54" s="25"/>
       <c r="C54" s="9"/>
       <c r="D54" s="9"/>
       <c r="E54" s="9"/>
@@ -2592,11 +2592,11 @@
       <c r="N54" s="9"/>
       <c r="O54" s="9"/>
       <c r="P54" s="9"/>
-      <c r="Q54" s="29"/>
+      <c r="Q54" s="25"/>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A55" s="29"/>
-      <c r="B55" s="29"/>
+      <c r="A55" s="25"/>
+      <c r="B55" s="25"/>
       <c r="C55" s="9"/>
       <c r="D55" s="9"/>
       <c r="E55" s="9"/>
@@ -2611,11 +2611,11 @@
       <c r="N55" s="9"/>
       <c r="O55" s="9"/>
       <c r="P55" s="9"/>
-      <c r="Q55" s="29"/>
+      <c r="Q55" s="25"/>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A56" s="29"/>
-      <c r="B56" s="29"/>
+      <c r="A56" s="25"/>
+      <c r="B56" s="25"/>
       <c r="C56" s="9"/>
       <c r="D56" s="9"/>
       <c r="E56" s="9"/>
@@ -2630,11 +2630,11 @@
       <c r="N56" s="9"/>
       <c r="O56" s="9"/>
       <c r="P56" s="9"/>
-      <c r="Q56" s="29"/>
+      <c r="Q56" s="25"/>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A57" s="29"/>
-      <c r="B57" s="29"/>
+      <c r="A57" s="25"/>
+      <c r="B57" s="25"/>
       <c r="C57" s="9"/>
       <c r="D57" s="9"/>
       <c r="E57" s="9"/>
@@ -2649,11 +2649,11 @@
       <c r="N57" s="9"/>
       <c r="O57" s="9"/>
       <c r="P57" s="9"/>
-      <c r="Q57" s="29"/>
+      <c r="Q57" s="25"/>
     </row>
     <row r="58" spans="1:17" ht="8.4499999999999993" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="29"/>
-      <c r="B58" s="29"/>
+      <c r="A58" s="25"/>
+      <c r="B58" s="25"/>
       <c r="C58" s="9"/>
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
@@ -2668,137 +2668,152 @@
       <c r="N58" s="9"/>
       <c r="O58" s="9"/>
       <c r="P58" s="9"/>
-      <c r="Q58" s="29"/>
+      <c r="Q58" s="25"/>
     </row>
     <row r="59" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="29"/>
-      <c r="B59" s="29"/>
-      <c r="C59" s="34" t="s">
+      <c r="A59" s="25"/>
+      <c r="B59" s="25"/>
+      <c r="C59" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D59" s="34"/>
-      <c r="E59" s="34"/>
-      <c r="F59" s="34"/>
-      <c r="G59" s="34"/>
-      <c r="H59" s="29"/>
-      <c r="I59" s="29"/>
-      <c r="J59" s="29"/>
-      <c r="K59" s="29"/>
-      <c r="L59" s="29"/>
-      <c r="M59" s="29"/>
-      <c r="N59" s="29"/>
-      <c r="O59" s="29"/>
-      <c r="P59" s="29"/>
-      <c r="Q59" s="29"/>
+      <c r="D59" s="31"/>
+      <c r="E59" s="31"/>
+      <c r="F59" s="31"/>
+      <c r="G59" s="31"/>
+      <c r="H59" s="25"/>
+      <c r="I59" s="25"/>
+      <c r="J59" s="25"/>
+      <c r="K59" s="25"/>
+      <c r="L59" s="25"/>
+      <c r="M59" s="25"/>
+      <c r="N59" s="25"/>
+      <c r="O59" s="25"/>
+      <c r="P59" s="25"/>
+      <c r="Q59" s="25"/>
     </row>
     <row r="60" spans="1:17" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="29"/>
-      <c r="B60" s="29"/>
-      <c r="C60" s="29"/>
-      <c r="D60" s="29"/>
-      <c r="E60" s="29"/>
-      <c r="F60" s="29"/>
-      <c r="G60" s="29"/>
-      <c r="H60" s="29"/>
-      <c r="I60" s="29"/>
-      <c r="J60" s="29"/>
-      <c r="K60" s="29"/>
-      <c r="L60" s="29"/>
-      <c r="M60" s="29"/>
-      <c r="N60" s="29"/>
-      <c r="O60" s="29"/>
-      <c r="P60" s="29"/>
-      <c r="Q60" s="29"/>
+      <c r="A60" s="25"/>
+      <c r="B60" s="25"/>
+      <c r="C60" s="25"/>
+      <c r="D60" s="25"/>
+      <c r="E60" s="25"/>
+      <c r="F60" s="25"/>
+      <c r="G60" s="25"/>
+      <c r="H60" s="25"/>
+      <c r="I60" s="25"/>
+      <c r="J60" s="25"/>
+      <c r="K60" s="25"/>
+      <c r="L60" s="25"/>
+      <c r="M60" s="25"/>
+      <c r="N60" s="25"/>
+      <c r="O60" s="25"/>
+      <c r="P60" s="25"/>
+      <c r="Q60" s="25"/>
     </row>
     <row r="61" spans="1:17" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="29"/>
-      <c r="B61" s="29"/>
-      <c r="C61" s="29"/>
-      <c r="D61" s="29"/>
-      <c r="E61" s="29"/>
-      <c r="F61" s="29"/>
-      <c r="G61" s="29"/>
-      <c r="H61" s="29"/>
-      <c r="I61" s="29"/>
-      <c r="J61" s="29"/>
-      <c r="K61" s="29"/>
-      <c r="L61" s="29"/>
-      <c r="M61" s="29"/>
-      <c r="N61" s="29"/>
-      <c r="O61" s="29"/>
-      <c r="P61" s="29"/>
-      <c r="Q61" s="29"/>
+      <c r="A61" s="25"/>
+      <c r="B61" s="25"/>
+      <c r="C61" s="25"/>
+      <c r="D61" s="25"/>
+      <c r="E61" s="25"/>
+      <c r="F61" s="25"/>
+      <c r="G61" s="25"/>
+      <c r="H61" s="25"/>
+      <c r="I61" s="25"/>
+      <c r="J61" s="25"/>
+      <c r="K61" s="25"/>
+      <c r="L61" s="25"/>
+      <c r="M61" s="25"/>
+      <c r="N61" s="25"/>
+      <c r="O61" s="25"/>
+      <c r="P61" s="25"/>
+      <c r="Q61" s="25"/>
     </row>
     <row r="62" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A62" s="29"/>
-      <c r="B62" s="29"/>
+      <c r="A62" s="25"/>
+      <c r="B62" s="25"/>
       <c r="C62" s="7" t="s">
         <v>48</v>
       </c>
       <c r="D62" s="23"/>
       <c r="E62" s="24"/>
-      <c r="G62" s="29"/>
-      <c r="H62" s="29"/>
-      <c r="I62" s="29"/>
-      <c r="J62" s="29"/>
-      <c r="K62" s="29"/>
-      <c r="L62" s="29"/>
-      <c r="M62" s="29"/>
-      <c r="N62" s="32" t="s">
+      <c r="G62" s="25"/>
+      <c r="H62" s="25"/>
+      <c r="I62" s="25"/>
+      <c r="J62" s="25"/>
+      <c r="K62" s="25"/>
+      <c r="L62" s="25"/>
+      <c r="M62" s="25"/>
+      <c r="N62" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="O62" s="32"/>
-      <c r="P62" s="32"/>
-      <c r="Q62" s="29"/>
+      <c r="O62" s="29"/>
+      <c r="P62" s="29"/>
+      <c r="Q62" s="25"/>
     </row>
     <row r="63" spans="1:17" ht="13.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="29"/>
-      <c r="B63" s="29"/>
-      <c r="C63" s="29"/>
-      <c r="D63" s="29"/>
-      <c r="E63" s="29"/>
-      <c r="F63" s="29"/>
-      <c r="G63" s="29"/>
-      <c r="H63" s="29"/>
-      <c r="I63" s="29"/>
-      <c r="J63" s="29"/>
-      <c r="K63" s="29"/>
-      <c r="L63" s="29"/>
-      <c r="M63" s="29"/>
-      <c r="N63" s="29"/>
-      <c r="O63" s="29"/>
-      <c r="P63" s="29"/>
-      <c r="Q63" s="29"/>
+      <c r="A63" s="25"/>
+      <c r="B63" s="25"/>
+      <c r="C63" s="25"/>
+      <c r="D63" s="25"/>
+      <c r="E63" s="25"/>
+      <c r="F63" s="25"/>
+      <c r="G63" s="25"/>
+      <c r="H63" s="25"/>
+      <c r="I63" s="25"/>
+      <c r="J63" s="25"/>
+      <c r="K63" s="25"/>
+      <c r="L63" s="25"/>
+      <c r="M63" s="25"/>
+      <c r="N63" s="25"/>
+      <c r="O63" s="25"/>
+      <c r="P63" s="25"/>
+      <c r="Q63" s="25"/>
     </row>
     <row r="64" spans="1:17" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="29"/>
-      <c r="C64" s="29"/>
-      <c r="D64" s="29"/>
-      <c r="E64" s="29"/>
-      <c r="F64" s="29"/>
-      <c r="G64" s="29"/>
-      <c r="H64" s="29"/>
-      <c r="I64" s="29"/>
-      <c r="J64" s="29"/>
-      <c r="K64" s="29"/>
-      <c r="L64" s="29"/>
-      <c r="M64" s="29"/>
-      <c r="N64" s="29"/>
-      <c r="O64" s="29"/>
-      <c r="P64" s="29"/>
-      <c r="Q64" s="29"/>
+      <c r="B64" s="25"/>
+      <c r="C64" s="25"/>
+      <c r="D64" s="25"/>
+      <c r="E64" s="25"/>
+      <c r="F64" s="25"/>
+      <c r="G64" s="25"/>
+      <c r="H64" s="25"/>
+      <c r="I64" s="25"/>
+      <c r="J64" s="25"/>
+      <c r="K64" s="25"/>
+      <c r="L64" s="25"/>
+      <c r="M64" s="25"/>
+      <c r="N64" s="25"/>
+      <c r="O64" s="25"/>
+      <c r="P64" s="25"/>
+      <c r="Q64" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="C42:P42"/>
-    <mergeCell ref="L29:P31"/>
-    <mergeCell ref="C23:P23"/>
-    <mergeCell ref="C25:P25"/>
-    <mergeCell ref="L35:P37"/>
-    <mergeCell ref="C34:P34"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="L26:O26"/>
+    <mergeCell ref="F6:J6"/>
+    <mergeCell ref="F7:J7"/>
+    <mergeCell ref="F14:J14"/>
+    <mergeCell ref="F22:J22"/>
+    <mergeCell ref="F35:J35"/>
+    <mergeCell ref="C15:P16"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="Q2:Q62"/>
+    <mergeCell ref="L22:P22"/>
+    <mergeCell ref="F27:P27"/>
+    <mergeCell ref="C10:J10"/>
+    <mergeCell ref="C2:L4"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="L6:P6"/>
+    <mergeCell ref="M4:P4"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="C60:P61"/>
+    <mergeCell ref="C32:P32"/>
+    <mergeCell ref="H59:P59"/>
+    <mergeCell ref="C18:P18"/>
+    <mergeCell ref="G62:M62"/>
+    <mergeCell ref="A2:A63"/>
     <mergeCell ref="B63:Q64"/>
     <mergeCell ref="C38:P38"/>
     <mergeCell ref="N62:P62"/>
@@ -2815,30 +2830,15 @@
     <mergeCell ref="H41:M41"/>
     <mergeCell ref="C5:P5"/>
     <mergeCell ref="F43:J43"/>
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="Q2:Q62"/>
-    <mergeCell ref="L22:P22"/>
-    <mergeCell ref="F27:P27"/>
-    <mergeCell ref="C10:J10"/>
-    <mergeCell ref="C2:L4"/>
-    <mergeCell ref="M3:P3"/>
-    <mergeCell ref="L6:P6"/>
-    <mergeCell ref="M4:P4"/>
-    <mergeCell ref="M2:P2"/>
-    <mergeCell ref="C60:P61"/>
-    <mergeCell ref="C32:P32"/>
-    <mergeCell ref="H59:P59"/>
-    <mergeCell ref="C18:P18"/>
-    <mergeCell ref="G62:M62"/>
-    <mergeCell ref="A2:A63"/>
-    <mergeCell ref="F6:J6"/>
-    <mergeCell ref="F7:J7"/>
-    <mergeCell ref="F14:J14"/>
-    <mergeCell ref="F22:J22"/>
-    <mergeCell ref="F35:J35"/>
-    <mergeCell ref="C15:P16"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C42:P42"/>
+    <mergeCell ref="L29:P31"/>
+    <mergeCell ref="C23:P23"/>
+    <mergeCell ref="C25:P25"/>
+    <mergeCell ref="L35:P37"/>
+    <mergeCell ref="C34:P34"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="L26:O26"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="81" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
fixed the print mismatch after converting to pdf
</commit_message>
<xml_diff>
--- a/core/main/templates/print_excel/cmf_template.xlsx
+++ b/core/main/templates/print_excel/cmf_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brant\VS Code Web\ColorMatch\core\main\templates\print_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{840B428F-DF6C-4563-8BC3-A84843E4ADA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C942C8-9BA7-487A-95DA-EB3CBBCF5783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -593,8 +593,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7904876" y="78581"/>
-          <a:ext cx="824" cy="9907086"/>
+          <a:off x="8248981" y="78581"/>
+          <a:ext cx="824" cy="9907839"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -2840,8 +2840,8 @@
     <mergeCell ref="O33:P33"/>
     <mergeCell ref="L26:O26"/>
   </mergeCells>
-  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="81" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="10001" scale="63" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
modified the template to merge the remarks
</commit_message>
<xml_diff>
--- a/core/main/templates/print_excel/cmf_template.xlsx
+++ b/core/main/templates/print_excel/cmf_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brant\VS Code Web\ColorMatch\core\main\templates\print_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{707B23E8-A445-43E3-BBBC-D949716DAEB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7873C01D-006F-4ACF-A389-C2FE8266A10C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3330" yWindow="930" windowWidth="16395" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REVISE CMF" sheetId="1" r:id="rId1"/>
@@ -297,7 +297,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -397,42 +397,45 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1457,105 +1460,105 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28"/>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
-      <c r="Q1" s="28"/>
+      <c r="A1" s="31"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
-      <c r="O2" s="28"/>
-      <c r="P2" s="28"/>
-      <c r="Q2" s="28"/>
+      <c r="A2" s="31"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="31"/>
     </row>
     <row r="3" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="28"/>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
-      <c r="K3" s="28"/>
-      <c r="L3" s="28"/>
-      <c r="M3" s="38" t="s">
+      <c r="A3" s="31"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="N3" s="38"/>
-      <c r="O3" s="38"/>
-      <c r="P3" s="38"/>
-      <c r="Q3" s="28"/>
+      <c r="N3" s="33"/>
+      <c r="O3" s="33"/>
+      <c r="P3" s="33"/>
+      <c r="Q3" s="31"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="28"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="28"/>
-      <c r="M4" s="28"/>
-      <c r="N4" s="28"/>
-      <c r="O4" s="28"/>
-      <c r="P4" s="28"/>
-      <c r="Q4" s="28"/>
+      <c r="A4" s="31"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="31"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="28"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="28"/>
-      <c r="P5" s="28"/>
-      <c r="Q5" s="28"/>
+      <c r="A5" s="31"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="31"/>
     </row>
     <row r="6" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="28"/>
-      <c r="B6" s="28"/>
+      <c r="A6" s="31"/>
+      <c r="B6" s="31"/>
       <c r="C6" s="1" t="s">
         <v>35</v>
       </c>
@@ -1563,22 +1566,22 @@
       <c r="E6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="29"/>
+      <c r="J6" s="29"/>
       <c r="K6" s="1"/>
-      <c r="L6" s="28"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28"/>
-      <c r="O6" s="28"/>
-      <c r="P6" s="28"/>
-      <c r="Q6" s="28"/>
+      <c r="L6" s="31"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="31"/>
+      <c r="O6" s="31"/>
+      <c r="P6" s="31"/>
+      <c r="Q6" s="31"/>
     </row>
     <row r="7" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="28"/>
-      <c r="B7" s="28"/>
+      <c r="A7" s="31"/>
+      <c r="B7" s="31"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1593,11 +1596,11 @@
       <c r="N7" s="11"/>
       <c r="O7" s="11"/>
       <c r="P7" s="11"/>
-      <c r="Q7" s="28"/>
+      <c r="Q7" s="31"/>
     </row>
     <row r="8" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="28"/>
-      <c r="B8" s="28"/>
+      <c r="A8" s="31"/>
+      <c r="B8" s="31"/>
       <c r="C8" s="6" t="s">
         <v>1</v>
       </c>
@@ -1605,22 +1608,22 @@
       <c r="E8" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="36"/>
-      <c r="J8" s="36"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="28"/>
       <c r="K8" s="12"/>
       <c r="L8" s="10"/>
       <c r="M8" s="10"/>
       <c r="N8" s="10"/>
       <c r="O8" s="10"/>
       <c r="P8" s="1"/>
-      <c r="Q8" s="28"/>
+      <c r="Q8" s="31"/>
     </row>
     <row r="9" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="28"/>
-      <c r="B9" s="28"/>
+      <c r="A9" s="31"/>
+      <c r="B9" s="31"/>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
@@ -1635,11 +1638,11 @@
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
-      <c r="Q9" s="28"/>
+      <c r="Q9" s="31"/>
     </row>
     <row r="10" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="28"/>
-      <c r="B10" s="28"/>
+      <c r="A10" s="31"/>
+      <c r="B10" s="31"/>
       <c r="C10" s="6" t="s">
         <v>2</v>
       </c>
@@ -1647,17 +1650,17 @@
       <c r="E10" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
-      <c r="J10" s="35"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37"/>
       <c r="K10" s="15"/>
-      <c r="Q10" s="28"/>
+      <c r="Q10" s="31"/>
     </row>
     <row r="11" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="28"/>
-      <c r="B11" s="28"/>
+      <c r="A11" s="31"/>
+      <c r="B11" s="31"/>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
@@ -1667,11 +1670,11 @@
       <c r="I11" s="15"/>
       <c r="J11" s="15"/>
       <c r="K11" s="15"/>
-      <c r="Q11" s="28"/>
+      <c r="Q11" s="31"/>
     </row>
     <row r="12" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="28"/>
-      <c r="B12" s="28"/>
+      <c r="A12" s="31"/>
+      <c r="B12" s="31"/>
       <c r="C12" s="6" t="s">
         <v>40</v>
       </c>
@@ -1679,17 +1682,17 @@
       <c r="E12" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37"/>
       <c r="K12" s="15"/>
-      <c r="Q12" s="28"/>
+      <c r="Q12" s="31"/>
     </row>
     <row r="13" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="28"/>
-      <c r="B13" s="28"/>
+      <c r="A13" s="31"/>
+      <c r="B13" s="31"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
       <c r="E13" s="11"/>
@@ -1699,11 +1702,11 @@
       <c r="I13" s="11"/>
       <c r="J13" s="11"/>
       <c r="K13" s="11"/>
-      <c r="Q13" s="28"/>
+      <c r="Q13" s="31"/>
     </row>
     <row r="14" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="28"/>
-      <c r="B14" s="28"/>
+      <c r="A14" s="31"/>
+      <c r="B14" s="31"/>
       <c r="C14" s="6" t="s">
         <v>3</v>
       </c>
@@ -1722,11 +1725,11 @@
         <v>9</v>
       </c>
       <c r="K14" s="1"/>
-      <c r="Q14" s="28"/>
+      <c r="Q14" s="31"/>
     </row>
     <row r="15" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="28"/>
-      <c r="B15" s="28"/>
+      <c r="A15" s="31"/>
+      <c r="B15" s="31"/>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
@@ -1735,11 +1738,11 @@
       <c r="I15" s="25"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
-      <c r="Q15" s="28"/>
+      <c r="Q15" s="31"/>
     </row>
     <row r="16" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="28"/>
-      <c r="B16" s="28"/>
+      <c r="A16" s="31"/>
+      <c r="B16" s="31"/>
       <c r="C16" s="6" t="s">
         <v>5</v>
       </c>
@@ -1747,22 +1750,22 @@
       <c r="E16" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F16" s="36"/>
-      <c r="G16" s="36"/>
-      <c r="H16" s="36"/>
-      <c r="I16" s="36"/>
-      <c r="J16" s="36"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="28"/>
       <c r="K16" s="12"/>
       <c r="L16" s="10"/>
       <c r="M16" s="10"/>
       <c r="N16" s="10"/>
       <c r="O16" s="10"/>
       <c r="P16" s="1"/>
-      <c r="Q16" s="28"/>
+      <c r="Q16" s="31"/>
     </row>
     <row r="17" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="28"/>
-      <c r="B17" s="28"/>
+      <c r="A17" s="31"/>
+      <c r="B17" s="31"/>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
@@ -1777,11 +1780,11 @@
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
-      <c r="Q17" s="28"/>
+      <c r="Q17" s="31"/>
     </row>
     <row r="18" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="28"/>
-      <c r="B18" s="28"/>
+      <c r="A18" s="31"/>
+      <c r="B18" s="31"/>
       <c r="C18" s="6" t="s">
         <v>6</v>
       </c>
@@ -1789,22 +1792,22 @@
       <c r="E18" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="36"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="28"/>
       <c r="K18" s="12"/>
       <c r="L18" s="10"/>
       <c r="M18" s="10"/>
       <c r="N18" s="10"/>
       <c r="O18" s="10"/>
       <c r="P18" s="1"/>
-      <c r="Q18" s="28"/>
+      <c r="Q18" s="31"/>
     </row>
     <row r="19" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="28"/>
-      <c r="B19" s="28"/>
+      <c r="A19" s="31"/>
+      <c r="B19" s="31"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
@@ -1819,11 +1822,11 @@
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
-      <c r="Q19" s="28"/>
+      <c r="Q19" s="31"/>
     </row>
     <row r="20" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="28"/>
-      <c r="B20" s="28"/>
+      <c r="A20" s="31"/>
+      <c r="B20" s="31"/>
       <c r="C20" s="6" t="s">
         <v>7</v>
       </c>
@@ -1831,41 +1834,41 @@
       <c r="E20" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F20" s="31"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="31"/>
-      <c r="J20" s="31"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
       <c r="K20" s="10"/>
       <c r="L20" s="10"/>
       <c r="M20" s="10"/>
       <c r="N20" s="10"/>
       <c r="O20" s="10"/>
       <c r="P20" s="1"/>
-      <c r="Q20" s="28"/>
+      <c r="Q20" s="31"/>
     </row>
     <row r="21" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="28"/>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="28"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="28"/>
-      <c r="L21" s="28"/>
-      <c r="M21" s="28"/>
-      <c r="N21" s="28"/>
-      <c r="O21" s="28"/>
-      <c r="P21" s="28"/>
-      <c r="Q21" s="28"/>
+      <c r="A21" s="31"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
+      <c r="L21" s="31"/>
+      <c r="M21" s="31"/>
+      <c r="N21" s="31"/>
+      <c r="O21" s="31"/>
+      <c r="P21" s="31"/>
+      <c r="Q21" s="31"/>
     </row>
     <row r="22" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="28"/>
-      <c r="B22" s="28"/>
+      <c r="A22" s="31"/>
+      <c r="B22" s="31"/>
       <c r="C22" s="6" t="s">
         <v>41</v>
       </c>
@@ -1892,30 +1895,30 @@
       <c r="M22" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="Q22" s="28"/>
+      <c r="Q22" s="31"/>
     </row>
     <row r="23" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="28"/>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="28"/>
-      <c r="K23" s="28"/>
-      <c r="L23" s="28"/>
-      <c r="M23" s="28"/>
-      <c r="N23" s="28"/>
-      <c r="O23" s="28"/>
-      <c r="P23" s="28"/>
-      <c r="Q23" s="28"/>
+      <c r="A23" s="31"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="31"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
+      <c r="L23" s="31"/>
+      <c r="M23" s="31"/>
+      <c r="N23" s="31"/>
+      <c r="O23" s="31"/>
+      <c r="P23" s="31"/>
+      <c r="Q23" s="31"/>
     </row>
     <row r="24" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="28"/>
-      <c r="B24" s="28"/>
+      <c r="A24" s="31"/>
+      <c r="B24" s="31"/>
       <c r="F24" s="14" t="b">
         <v>0</v>
       </c>
@@ -1935,38 +1938,38 @@
       <c r="M24" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q24" s="28"/>
+      <c r="Q24" s="31"/>
     </row>
     <row r="25" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="28"/>
-      <c r="B25" s="28"/>
+      <c r="A25" s="31"/>
+      <c r="B25" s="31"/>
       <c r="G25" s="1"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
       <c r="M25" s="1"/>
-      <c r="Q25" s="28"/>
+      <c r="Q25" s="31"/>
     </row>
     <row r="26" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="28"/>
-      <c r="B26" s="28"/>
+      <c r="A26" s="31"/>
+      <c r="B26" s="31"/>
       <c r="F26" s="20" t="b">
         <v>0</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H26" s="37"/>
-      <c r="I26" s="37"/>
-      <c r="J26" s="37"/>
-      <c r="K26" s="37"/>
-      <c r="L26" s="37"/>
-      <c r="M26" s="37"/>
-      <c r="N26" s="37"/>
-      <c r="Q26" s="28"/>
+      <c r="H26" s="38"/>
+      <c r="I26" s="38"/>
+      <c r="J26" s="38"/>
+      <c r="K26" s="38"/>
+      <c r="L26" s="38"/>
+      <c r="M26" s="38"/>
+      <c r="N26" s="38"/>
+      <c r="Q26" s="31"/>
     </row>
     <row r="27" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="28"/>
-      <c r="B27" s="28"/>
+      <c r="A27" s="31"/>
+      <c r="B27" s="31"/>
       <c r="F27" s="26"/>
       <c r="G27" s="1"/>
       <c r="H27" s="24"/>
@@ -1976,57 +1979,57 @@
       <c r="L27" s="24"/>
       <c r="M27" s="24"/>
       <c r="N27" s="24"/>
-      <c r="Q27" s="28"/>
+      <c r="Q27" s="31"/>
     </row>
     <row r="28" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="28"/>
-      <c r="B28" s="28"/>
-      <c r="C28" s="40" t="s">
+      <c r="A28" s="31"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="D28" s="40"/>
+      <c r="D28" s="32"/>
       <c r="E28" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="31"/>
-      <c r="I28" s="31"/>
-      <c r="J28" s="31"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="29"/>
+      <c r="J28" s="29"/>
       <c r="K28" s="1"/>
-      <c r="L28" s="28"/>
-      <c r="M28" s="28"/>
-      <c r="N28" s="28"/>
-      <c r="O28" s="28"/>
-      <c r="P28" s="28"/>
-      <c r="Q28" s="28"/>
+      <c r="L28" s="31"/>
+      <c r="M28" s="31"/>
+      <c r="N28" s="31"/>
+      <c r="O28" s="31"/>
+      <c r="P28" s="31"/>
+      <c r="Q28" s="31"/>
     </row>
     <row r="29" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="28"/>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="28"/>
-      <c r="M29" s="28"/>
-      <c r="N29" s="28"/>
-      <c r="O29" s="28"/>
-      <c r="P29" s="28"/>
-      <c r="Q29" s="28"/>
+      <c r="A29" s="31"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="31"/>
+      <c r="J29" s="31"/>
+      <c r="K29" s="31"/>
+      <c r="L29" s="31"/>
+      <c r="M29" s="31"/>
+      <c r="N29" s="31"/>
+      <c r="O29" s="31"/>
+      <c r="P29" s="31"/>
+      <c r="Q29" s="31"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="28"/>
-      <c r="B30" s="28"/>
-      <c r="C30" s="40" t="s">
+      <c r="A30" s="31"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="D30" s="40"/>
+      <c r="D30" s="32"/>
       <c r="E30" s="2" t="s">
         <v>4</v>
       </c>
@@ -2049,32 +2052,32 @@
       <c r="N30" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="O30" s="28"/>
-      <c r="P30" s="28"/>
-      <c r="Q30" s="28"/>
+      <c r="O30" s="31"/>
+      <c r="P30" s="31"/>
+      <c r="Q30" s="31"/>
     </row>
     <row r="31" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="28"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="28"/>
-      <c r="K31" s="28"/>
-      <c r="L31" s="28"/>
-      <c r="M31" s="28"/>
-      <c r="N31" s="28"/>
-      <c r="O31" s="28"/>
-      <c r="P31" s="28"/>
-      <c r="Q31" s="28"/>
+      <c r="A31" s="31"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="31"/>
+      <c r="F31" s="31"/>
+      <c r="G31" s="31"/>
+      <c r="H31" s="31"/>
+      <c r="I31" s="31"/>
+      <c r="J31" s="31"/>
+      <c r="K31" s="31"/>
+      <c r="L31" s="31"/>
+      <c r="M31" s="31"/>
+      <c r="N31" s="31"/>
+      <c r="O31" s="31"/>
+      <c r="P31" s="31"/>
+      <c r="Q31" s="31"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="28"/>
-      <c r="B32" s="28"/>
+      <c r="A32" s="31"/>
+      <c r="B32" s="31"/>
       <c r="F32" s="19" t="b">
         <v>0</v>
       </c>
@@ -2088,31 +2091,31 @@
         <v>38</v>
       </c>
       <c r="K32" s="1"/>
-      <c r="L32" s="31"/>
-      <c r="M32" s="31"/>
-      <c r="N32" s="31"/>
-      <c r="O32" s="31"/>
-      <c r="Q32" s="28"/>
+      <c r="L32" s="29"/>
+      <c r="M32" s="29"/>
+      <c r="N32" s="29"/>
+      <c r="O32" s="29"/>
+      <c r="Q32" s="31"/>
     </row>
     <row r="33" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="28"/>
-      <c r="B33" s="28"/>
-      <c r="F33" s="28"/>
-      <c r="G33" s="28"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="28"/>
-      <c r="K33" s="28"/>
-      <c r="L33" s="28"/>
-      <c r="M33" s="28"/>
-      <c r="N33" s="28"/>
-      <c r="O33" s="28"/>
-      <c r="P33" s="28"/>
-      <c r="Q33" s="28"/>
+      <c r="A33" s="31"/>
+      <c r="B33" s="31"/>
+      <c r="F33" s="31"/>
+      <c r="G33" s="31"/>
+      <c r="H33" s="31"/>
+      <c r="I33" s="31"/>
+      <c r="J33" s="31"/>
+      <c r="K33" s="31"/>
+      <c r="L33" s="31"/>
+      <c r="M33" s="31"/>
+      <c r="N33" s="31"/>
+      <c r="O33" s="31"/>
+      <c r="P33" s="31"/>
+      <c r="Q33" s="31"/>
     </row>
     <row r="34" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="28"/>
-      <c r="B34" s="28"/>
+      <c r="A34" s="31"/>
+      <c r="B34" s="31"/>
       <c r="C34" s="6" t="s">
         <v>20</v>
       </c>
@@ -2120,22 +2123,22 @@
       <c r="E34" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F34" s="36"/>
-      <c r="G34" s="36"/>
-      <c r="H34" s="36"/>
-      <c r="I34" s="36"/>
-      <c r="J34" s="36"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="28"/>
+      <c r="H34" s="28"/>
+      <c r="I34" s="28"/>
+      <c r="J34" s="28"/>
       <c r="K34" s="13"/>
       <c r="L34" s="3"/>
       <c r="M34" s="4"/>
       <c r="N34" s="4"/>
       <c r="O34" s="4"/>
       <c r="P34" s="4"/>
-      <c r="Q34" s="28"/>
+      <c r="Q34" s="31"/>
     </row>
     <row r="35" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="28"/>
-      <c r="B35" s="28"/>
+      <c r="A35" s="31"/>
+      <c r="B35" s="31"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
       <c r="E35" s="1"/>
@@ -2150,11 +2153,11 @@
       <c r="N35" s="4"/>
       <c r="O35" s="4"/>
       <c r="P35" s="4"/>
-      <c r="Q35" s="28"/>
+      <c r="Q35" s="31"/>
     </row>
     <row r="36" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="28"/>
-      <c r="B36" s="28"/>
+      <c r="A36" s="31"/>
+      <c r="B36" s="31"/>
       <c r="C36" s="6" t="s">
         <v>44</v>
       </c>
@@ -2175,18 +2178,18 @@
         <v>22</v>
       </c>
       <c r="K36" s="1"/>
-      <c r="L36" s="29" t="s">
+      <c r="L36" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="M36" s="29"/>
-      <c r="N36" s="29"/>
-      <c r="O36" s="29"/>
-      <c r="P36" s="29"/>
-      <c r="Q36" s="28"/>
+      <c r="M36" s="39"/>
+      <c r="N36" s="39"/>
+      <c r="O36" s="39"/>
+      <c r="P36" s="39"/>
+      <c r="Q36" s="31"/>
     </row>
     <row r="37" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="28"/>
-      <c r="B37" s="28"/>
+      <c r="A37" s="31"/>
+      <c r="B37" s="31"/>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
       <c r="E37" s="1"/>
@@ -2195,16 +2198,16 @@
       <c r="I37" s="23"/>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
-      <c r="L37" s="29"/>
-      <c r="M37" s="29"/>
-      <c r="N37" s="29"/>
-      <c r="O37" s="29"/>
-      <c r="P37" s="29"/>
-      <c r="Q37" s="28"/>
+      <c r="L37" s="39"/>
+      <c r="M37" s="39"/>
+      <c r="N37" s="39"/>
+      <c r="O37" s="39"/>
+      <c r="P37" s="39"/>
+      <c r="Q37" s="31"/>
     </row>
     <row r="38" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="28"/>
-      <c r="B38" s="28"/>
+      <c r="A38" s="31"/>
+      <c r="B38" s="31"/>
       <c r="C38" s="6" t="s">
         <v>45</v>
       </c>
@@ -2212,22 +2215,22 @@
       <c r="E38" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F38" s="36"/>
-      <c r="G38" s="36"/>
-      <c r="H38" s="36"/>
-      <c r="I38" s="36"/>
-      <c r="J38" s="36"/>
+      <c r="F38" s="28"/>
+      <c r="G38" s="28"/>
+      <c r="H38" s="28"/>
+      <c r="I38" s="28"/>
+      <c r="J38" s="28"/>
       <c r="K38" s="13"/>
-      <c r="L38" s="29"/>
-      <c r="M38" s="29"/>
-      <c r="N38" s="29"/>
-      <c r="O38" s="29"/>
-      <c r="P38" s="29"/>
-      <c r="Q38" s="28"/>
+      <c r="L38" s="39"/>
+      <c r="M38" s="39"/>
+      <c r="N38" s="39"/>
+      <c r="O38" s="39"/>
+      <c r="P38" s="39"/>
+      <c r="Q38" s="31"/>
     </row>
     <row r="39" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="28"/>
-      <c r="B39" s="28"/>
+      <c r="A39" s="31"/>
+      <c r="B39" s="31"/>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
       <c r="E39" s="1"/>
@@ -2237,16 +2240,16 @@
       <c r="I39" s="13"/>
       <c r="J39" s="13"/>
       <c r="K39" s="13"/>
-      <c r="L39" s="29"/>
-      <c r="M39" s="29"/>
-      <c r="N39" s="29"/>
-      <c r="O39" s="29"/>
-      <c r="P39" s="29"/>
-      <c r="Q39" s="28"/>
+      <c r="L39" s="39"/>
+      <c r="M39" s="39"/>
+      <c r="N39" s="39"/>
+      <c r="O39" s="39"/>
+      <c r="P39" s="39"/>
+      <c r="Q39" s="31"/>
     </row>
     <row r="40" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="28"/>
-      <c r="B40" s="28"/>
+      <c r="A40" s="31"/>
+      <c r="B40" s="31"/>
       <c r="C40" s="1" t="s">
         <v>31</v>
       </c>
@@ -2267,35 +2270,35 @@
         <v>22</v>
       </c>
       <c r="K40" s="1"/>
-      <c r="L40" s="29"/>
-      <c r="M40" s="29"/>
-      <c r="N40" s="29"/>
-      <c r="O40" s="29"/>
-      <c r="P40" s="29"/>
-      <c r="Q40" s="28"/>
+      <c r="L40" s="39"/>
+      <c r="M40" s="39"/>
+      <c r="N40" s="39"/>
+      <c r="O40" s="39"/>
+      <c r="P40" s="39"/>
+      <c r="Q40" s="31"/>
     </row>
     <row r="41" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="28"/>
-      <c r="B41" s="28"/>
-      <c r="C41" s="28"/>
-      <c r="D41" s="28"/>
-      <c r="E41" s="28"/>
-      <c r="F41" s="28"/>
-      <c r="G41" s="28"/>
-      <c r="H41" s="28"/>
-      <c r="I41" s="28"/>
-      <c r="J41" s="28"/>
-      <c r="K41" s="28"/>
-      <c r="L41" s="28"/>
-      <c r="M41" s="28"/>
-      <c r="N41" s="28"/>
-      <c r="O41" s="28"/>
-      <c r="P41" s="28"/>
-      <c r="Q41" s="28"/>
+      <c r="A41" s="31"/>
+      <c r="B41" s="31"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="31"/>
+      <c r="E41" s="31"/>
+      <c r="F41" s="31"/>
+      <c r="G41" s="31"/>
+      <c r="H41" s="31"/>
+      <c r="I41" s="31"/>
+      <c r="J41" s="31"/>
+      <c r="K41" s="31"/>
+      <c r="L41" s="31"/>
+      <c r="M41" s="31"/>
+      <c r="N41" s="31"/>
+      <c r="O41" s="31"/>
+      <c r="P41" s="31"/>
+      <c r="Q41" s="31"/>
     </row>
     <row r="42" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="28"/>
-      <c r="B42" s="28"/>
+      <c r="A42" s="31"/>
+      <c r="B42" s="31"/>
       <c r="C42" s="6" t="s">
         <v>23</v>
       </c>
@@ -2322,32 +2325,32 @@
       <c r="M42" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="O42" s="31"/>
-      <c r="P42" s="31"/>
-      <c r="Q42" s="28"/>
+      <c r="O42" s="29"/>
+      <c r="P42" s="29"/>
+      <c r="Q42" s="31"/>
     </row>
     <row r="43" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="28"/>
-      <c r="B43" s="28"/>
-      <c r="C43" s="28"/>
-      <c r="D43" s="28"/>
-      <c r="E43" s="28"/>
-      <c r="F43" s="28"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="28"/>
-      <c r="I43" s="28"/>
-      <c r="J43" s="28"/>
-      <c r="K43" s="28"/>
-      <c r="L43" s="28"/>
-      <c r="M43" s="28"/>
-      <c r="N43" s="28"/>
-      <c r="O43" s="28"/>
-      <c r="P43" s="28"/>
-      <c r="Q43" s="28"/>
+      <c r="A43" s="31"/>
+      <c r="B43" s="31"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="31"/>
+      <c r="E43" s="31"/>
+      <c r="F43" s="31"/>
+      <c r="G43" s="31"/>
+      <c r="H43" s="31"/>
+      <c r="I43" s="31"/>
+      <c r="J43" s="31"/>
+      <c r="K43" s="31"/>
+      <c r="L43" s="31"/>
+      <c r="M43" s="31"/>
+      <c r="N43" s="31"/>
+      <c r="O43" s="31"/>
+      <c r="P43" s="31"/>
+      <c r="Q43" s="31"/>
     </row>
     <row r="44" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="28"/>
-      <c r="B44" s="28"/>
+      <c r="A44" s="31"/>
+      <c r="B44" s="31"/>
       <c r="C44" s="7" t="s">
         <v>36</v>
       </c>
@@ -2355,32 +2358,32 @@
       <c r="E44" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F44" s="39"/>
-      <c r="G44" s="39"/>
-      <c r="H44" s="39"/>
-      <c r="I44" s="39"/>
-      <c r="J44" s="39"/>
+      <c r="F44" s="30"/>
+      <c r="G44" s="30"/>
+      <c r="H44" s="30"/>
+      <c r="I44" s="30"/>
+      <c r="J44" s="30"/>
       <c r="K44" s="16"/>
-      <c r="L44" s="30"/>
-      <c r="M44" s="30"/>
-      <c r="N44" s="30"/>
-      <c r="O44" s="30"/>
-      <c r="P44" s="30"/>
-      <c r="Q44" s="28"/>
+      <c r="L44" s="40"/>
+      <c r="M44" s="40"/>
+      <c r="N44" s="40"/>
+      <c r="O44" s="40"/>
+      <c r="P44" s="40"/>
+      <c r="Q44" s="31"/>
     </row>
     <row r="45" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="28"/>
-      <c r="B45" s="28"/>
-      <c r="L45" s="30"/>
-      <c r="M45" s="30"/>
-      <c r="N45" s="30"/>
-      <c r="O45" s="30"/>
-      <c r="P45" s="30"/>
-      <c r="Q45" s="28"/>
+      <c r="A45" s="31"/>
+      <c r="B45" s="31"/>
+      <c r="L45" s="40"/>
+      <c r="M45" s="40"/>
+      <c r="N45" s="40"/>
+      <c r="O45" s="40"/>
+      <c r="P45" s="40"/>
+      <c r="Q45" s="31"/>
     </row>
     <row r="46" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" s="28"/>
-      <c r="B46" s="28"/>
+      <c r="A46" s="31"/>
+      <c r="B46" s="31"/>
       <c r="C46" s="1" t="s">
         <v>26</v>
       </c>
@@ -2401,35 +2404,35 @@
         <v>22</v>
       </c>
       <c r="K46" s="1"/>
-      <c r="L46" s="30"/>
-      <c r="M46" s="30"/>
-      <c r="N46" s="30"/>
-      <c r="O46" s="30"/>
-      <c r="P46" s="30"/>
-      <c r="Q46" s="28"/>
+      <c r="L46" s="40"/>
+      <c r="M46" s="40"/>
+      <c r="N46" s="40"/>
+      <c r="O46" s="40"/>
+      <c r="P46" s="40"/>
+      <c r="Q46" s="31"/>
     </row>
     <row r="47" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="28"/>
-      <c r="B47" s="28"/>
-      <c r="C47" s="28"/>
-      <c r="D47" s="28"/>
-      <c r="E47" s="28"/>
-      <c r="F47" s="28"/>
-      <c r="G47" s="28"/>
-      <c r="H47" s="28"/>
-      <c r="I47" s="28"/>
-      <c r="J47" s="28"/>
-      <c r="K47" s="28"/>
-      <c r="L47" s="28"/>
-      <c r="M47" s="28"/>
-      <c r="N47" s="28"/>
-      <c r="O47" s="28"/>
-      <c r="P47" s="28"/>
-      <c r="Q47" s="28"/>
+      <c r="A47" s="31"/>
+      <c r="B47" s="31"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="31"/>
+      <c r="E47" s="31"/>
+      <c r="F47" s="31"/>
+      <c r="G47" s="31"/>
+      <c r="H47" s="31"/>
+      <c r="I47" s="31"/>
+      <c r="J47" s="31"/>
+      <c r="K47" s="31"/>
+      <c r="L47" s="31"/>
+      <c r="M47" s="31"/>
+      <c r="N47" s="31"/>
+      <c r="O47" s="31"/>
+      <c r="P47" s="31"/>
+      <c r="Q47" s="31"/>
     </row>
     <row r="48" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A48" s="28"/>
-      <c r="B48" s="28"/>
+      <c r="A48" s="31"/>
+      <c r="B48" s="31"/>
       <c r="C48" s="6" t="s">
         <v>27</v>
       </c>
@@ -2450,11 +2453,11 @@
         <v>29</v>
       </c>
       <c r="K48" s="1"/>
-      <c r="Q48" s="28"/>
+      <c r="Q48" s="31"/>
     </row>
     <row r="49" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="28"/>
-      <c r="B49" s="28"/>
+      <c r="A49" s="31"/>
+      <c r="B49" s="31"/>
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
@@ -2464,11 +2467,11 @@
       <c r="K49" s="1"/>
       <c r="N49" s="1"/>
       <c r="P49" s="1"/>
-      <c r="Q49" s="28"/>
+      <c r="Q49" s="31"/>
     </row>
     <row r="50" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="28"/>
-      <c r="B50" s="28"/>
+      <c r="A50" s="31"/>
+      <c r="B50" s="31"/>
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
       <c r="E50" s="1"/>
@@ -2478,38 +2481,38 @@
       <c r="G50" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H50" s="37"/>
-      <c r="I50" s="37"/>
-      <c r="J50" s="37"/>
-      <c r="K50" s="37"/>
-      <c r="L50" s="37"/>
-      <c r="M50" s="37"/>
+      <c r="H50" s="38"/>
+      <c r="I50" s="38"/>
+      <c r="J50" s="38"/>
+      <c r="K50" s="38"/>
+      <c r="L50" s="38"/>
+      <c r="M50" s="38"/>
       <c r="N50" s="1"/>
       <c r="P50" s="1"/>
-      <c r="Q50" s="28"/>
+      <c r="Q50" s="31"/>
     </row>
     <row r="51" spans="1:17" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="28"/>
-      <c r="B51" s="28"/>
-      <c r="C51" s="28"/>
-      <c r="D51" s="28"/>
-      <c r="E51" s="28"/>
-      <c r="F51" s="28"/>
-      <c r="G51" s="28"/>
-      <c r="H51" s="28"/>
-      <c r="I51" s="28"/>
-      <c r="J51" s="28"/>
-      <c r="K51" s="28"/>
-      <c r="L51" s="28"/>
-      <c r="M51" s="28"/>
-      <c r="N51" s="28"/>
-      <c r="O51" s="28"/>
-      <c r="P51" s="28"/>
-      <c r="Q51" s="28"/>
+      <c r="A51" s="31"/>
+      <c r="B51" s="31"/>
+      <c r="C51" s="31"/>
+      <c r="D51" s="31"/>
+      <c r="E51" s="31"/>
+      <c r="F51" s="31"/>
+      <c r="G51" s="31"/>
+      <c r="H51" s="31"/>
+      <c r="I51" s="31"/>
+      <c r="J51" s="31"/>
+      <c r="K51" s="31"/>
+      <c r="L51" s="31"/>
+      <c r="M51" s="31"/>
+      <c r="N51" s="31"/>
+      <c r="O51" s="31"/>
+      <c r="P51" s="31"/>
+      <c r="Q51" s="31"/>
     </row>
     <row r="52" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="28"/>
-      <c r="B52" s="28"/>
+      <c r="A52" s="31"/>
+      <c r="B52" s="31"/>
       <c r="C52" s="6" t="s">
         <v>30</v>
       </c>
@@ -2517,22 +2520,22 @@
       <c r="E52" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F52" s="36"/>
-      <c r="G52" s="36"/>
-      <c r="H52" s="36"/>
-      <c r="I52" s="36"/>
-      <c r="J52" s="36"/>
+      <c r="F52" s="28"/>
+      <c r="G52" s="28"/>
+      <c r="H52" s="28"/>
+      <c r="I52" s="28"/>
+      <c r="J52" s="28"/>
       <c r="K52" s="13"/>
-      <c r="L52" s="33"/>
-      <c r="M52" s="33"/>
-      <c r="N52" s="33"/>
-      <c r="O52" s="33"/>
-      <c r="P52" s="33"/>
-      <c r="Q52" s="28"/>
+      <c r="L52" s="35"/>
+      <c r="M52" s="35"/>
+      <c r="N52" s="35"/>
+      <c r="O52" s="35"/>
+      <c r="P52" s="35"/>
+      <c r="Q52" s="31"/>
     </row>
     <row r="53" spans="1:17" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="28"/>
-      <c r="B53" s="28"/>
+      <c r="A53" s="31"/>
+      <c r="B53" s="31"/>
       <c r="C53" s="6"/>
       <c r="D53" s="6"/>
       <c r="E53" s="6"/>
@@ -2547,11 +2550,11 @@
       <c r="N53" s="13"/>
       <c r="O53" s="13"/>
       <c r="P53" s="13"/>
-      <c r="Q53" s="28"/>
+      <c r="Q53" s="31"/>
     </row>
     <row r="54" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="28"/>
-      <c r="B54" s="28"/>
+      <c r="A54" s="31"/>
+      <c r="B54" s="31"/>
       <c r="C54" s="6" t="s">
         <v>46</v>
       </c>
@@ -2578,11 +2581,11 @@
       <c r="N54" s="5"/>
       <c r="O54" s="5"/>
       <c r="P54" s="5"/>
-      <c r="Q54" s="28"/>
+      <c r="Q54" s="31"/>
     </row>
     <row r="55" spans="1:17" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="28"/>
-      <c r="B55" s="28"/>
+      <c r="A55" s="31"/>
+      <c r="B55" s="31"/>
       <c r="C55" s="6"/>
       <c r="D55" s="6"/>
       <c r="E55" s="1"/>
@@ -2597,11 +2600,11 @@
       <c r="N55" s="5"/>
       <c r="O55" s="5"/>
       <c r="P55" s="5"/>
-      <c r="Q55" s="28"/>
+      <c r="Q55" s="31"/>
     </row>
     <row r="56" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A56" s="28"/>
-      <c r="B56" s="28"/>
+      <c r="A56" s="31"/>
+      <c r="B56" s="31"/>
       <c r="C56" s="6" t="s">
         <v>47</v>
       </c>
@@ -2609,11 +2612,11 @@
       <c r="E56" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="Q56" s="28"/>
+      <c r="Q56" s="31"/>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A57" s="28"/>
-      <c r="B57" s="28"/>
+      <c r="A57" s="31"/>
+      <c r="B57" s="31"/>
       <c r="C57" s="8" t="s">
         <v>33</v>
       </c>
@@ -2630,11 +2633,11 @@
       <c r="N57" s="9"/>
       <c r="O57" s="9"/>
       <c r="P57" s="9"/>
-      <c r="Q57" s="28"/>
+      <c r="Q57" s="31"/>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A58" s="28"/>
-      <c r="B58" s="28"/>
+      <c r="A58" s="31"/>
+      <c r="B58" s="31"/>
       <c r="C58" s="9"/>
       <c r="D58" s="9"/>
       <c r="E58" s="9"/>
@@ -2649,180 +2652,182 @@
       <c r="N58" s="9"/>
       <c r="O58" s="9"/>
       <c r="P58" s="9"/>
-      <c r="Q58" s="28"/>
+      <c r="Q58" s="31"/>
     </row>
     <row r="59" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A59" s="28"/>
-      <c r="B59" s="28"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
-      <c r="G59" s="9"/>
-      <c r="H59" s="9"/>
-      <c r="I59" s="9"/>
-      <c r="J59" s="9"/>
-      <c r="K59" s="9"/>
-      <c r="L59" s="9"/>
-      <c r="M59" s="9"/>
-      <c r="N59" s="9"/>
-      <c r="O59" s="9"/>
+      <c r="A59" s="31"/>
+      <c r="B59" s="31"/>
+      <c r="C59" s="41"/>
+      <c r="D59" s="41"/>
+      <c r="E59" s="41"/>
+      <c r="F59" s="41"/>
+      <c r="G59" s="41"/>
+      <c r="H59" s="41"/>
+      <c r="I59" s="41"/>
+      <c r="J59" s="41"/>
+      <c r="K59" s="41"/>
+      <c r="L59" s="41"/>
+      <c r="M59" s="41"/>
+      <c r="N59" s="41"/>
+      <c r="O59" s="41"/>
       <c r="P59" s="9"/>
-      <c r="Q59" s="28"/>
+      <c r="Q59" s="31"/>
     </row>
     <row r="60" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A60" s="28"/>
-      <c r="B60" s="28"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9"/>
-      <c r="G60" s="9"/>
-      <c r="H60" s="9"/>
-      <c r="I60" s="9"/>
-      <c r="J60" s="9"/>
-      <c r="K60" s="9"/>
-      <c r="L60" s="9"/>
-      <c r="M60" s="9"/>
-      <c r="N60" s="9"/>
-      <c r="O60" s="9"/>
+      <c r="A60" s="31"/>
+      <c r="B60" s="31"/>
+      <c r="C60" s="41"/>
+      <c r="D60" s="41"/>
+      <c r="E60" s="41"/>
+      <c r="F60" s="41"/>
+      <c r="G60" s="41"/>
+      <c r="H60" s="41"/>
+      <c r="I60" s="41"/>
+      <c r="J60" s="41"/>
+      <c r="K60" s="41"/>
+      <c r="L60" s="41"/>
+      <c r="M60" s="41"/>
+      <c r="N60" s="41"/>
+      <c r="O60" s="41"/>
       <c r="P60" s="9"/>
-      <c r="Q60" s="28"/>
+      <c r="Q60" s="31"/>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A61" s="28"/>
-      <c r="B61" s="28"/>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="9"/>
-      <c r="F61" s="9"/>
-      <c r="G61" s="9"/>
-      <c r="H61" s="9"/>
-      <c r="I61" s="9"/>
-      <c r="J61" s="9"/>
-      <c r="K61" s="9"/>
-      <c r="L61" s="9"/>
-      <c r="M61" s="9"/>
-      <c r="N61" s="9"/>
-      <c r="O61" s="9"/>
+      <c r="A61" s="31"/>
+      <c r="B61" s="31"/>
+      <c r="C61" s="41"/>
+      <c r="D61" s="41"/>
+      <c r="E61" s="41"/>
+      <c r="F61" s="41"/>
+      <c r="G61" s="41"/>
+      <c r="H61" s="41"/>
+      <c r="I61" s="41"/>
+      <c r="J61" s="41"/>
+      <c r="K61" s="41"/>
+      <c r="L61" s="41"/>
+      <c r="M61" s="41"/>
+      <c r="N61" s="41"/>
+      <c r="O61" s="41"/>
       <c r="P61" s="9"/>
-      <c r="Q61" s="28"/>
+      <c r="Q61" s="31"/>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A62" s="28"/>
-      <c r="B62" s="28"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="9"/>
-      <c r="F62" s="9"/>
-      <c r="G62" s="9"/>
-      <c r="H62" s="9"/>
-      <c r="I62" s="9"/>
-      <c r="J62" s="9"/>
-      <c r="K62" s="9"/>
-      <c r="L62" s="9"/>
-      <c r="M62" s="9"/>
-      <c r="N62" s="9"/>
-      <c r="O62" s="9"/>
+      <c r="A62" s="31"/>
+      <c r="B62" s="31"/>
+      <c r="C62" s="41"/>
+      <c r="D62" s="41"/>
+      <c r="E62" s="41"/>
+      <c r="F62" s="41"/>
+      <c r="G62" s="41"/>
+      <c r="H62" s="41"/>
+      <c r="I62" s="41"/>
+      <c r="J62" s="41"/>
+      <c r="K62" s="41"/>
+      <c r="L62" s="41"/>
+      <c r="M62" s="41"/>
+      <c r="N62" s="41"/>
+      <c r="O62" s="41"/>
       <c r="P62" s="9"/>
-      <c r="Q62" s="28"/>
+      <c r="Q62" s="31"/>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A63" s="28"/>
-      <c r="B63" s="28"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
-      <c r="E63" s="9"/>
-      <c r="F63" s="9"/>
-      <c r="G63" s="9"/>
-      <c r="H63" s="9"/>
-      <c r="I63" s="9"/>
-      <c r="J63" s="9"/>
-      <c r="K63" s="9"/>
-      <c r="L63" s="9"/>
-      <c r="M63" s="9"/>
-      <c r="N63" s="9"/>
-      <c r="O63" s="9"/>
+      <c r="A63" s="31"/>
+      <c r="B63" s="31"/>
+      <c r="C63" s="41"/>
+      <c r="D63" s="41"/>
+      <c r="E63" s="41"/>
+      <c r="F63" s="41"/>
+      <c r="G63" s="41"/>
+      <c r="H63" s="41"/>
+      <c r="I63" s="41"/>
+      <c r="J63" s="41"/>
+      <c r="K63" s="41"/>
+      <c r="L63" s="41"/>
+      <c r="M63" s="41"/>
+      <c r="N63" s="41"/>
+      <c r="O63" s="41"/>
       <c r="P63" s="9"/>
-      <c r="Q63" s="28"/>
+      <c r="Q63" s="31"/>
     </row>
     <row r="64" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="28"/>
-      <c r="B64" s="28"/>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="9"/>
-      <c r="F64" s="9"/>
-      <c r="G64" s="9"/>
-      <c r="H64" s="9"/>
-      <c r="I64" s="9"/>
-      <c r="J64" s="9"/>
-      <c r="K64" s="9"/>
-      <c r="L64" s="9"/>
-      <c r="M64" s="9"/>
-      <c r="N64" s="9"/>
-      <c r="O64" s="9"/>
+      <c r="A64" s="31"/>
+      <c r="B64" s="31"/>
+      <c r="C64" s="41"/>
+      <c r="D64" s="41"/>
+      <c r="E64" s="41"/>
+      <c r="F64" s="41"/>
+      <c r="G64" s="41"/>
+      <c r="H64" s="41"/>
+      <c r="I64" s="41"/>
+      <c r="J64" s="41"/>
+      <c r="K64" s="41"/>
+      <c r="L64" s="41"/>
+      <c r="M64" s="41"/>
+      <c r="N64" s="41"/>
+      <c r="O64" s="41"/>
       <c r="P64" s="9"/>
-      <c r="Q64" s="28"/>
+      <c r="Q64" s="31"/>
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A65" s="28"/>
-      <c r="B65" s="28"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="9"/>
-      <c r="F65" s="9"/>
-      <c r="G65" s="9"/>
-      <c r="H65" s="9"/>
-      <c r="I65" s="9"/>
-      <c r="J65" s="9"/>
-      <c r="K65" s="9"/>
-      <c r="L65" s="9"/>
-      <c r="M65" s="9"/>
-      <c r="N65" s="9"/>
-      <c r="O65" s="9"/>
+      <c r="A65" s="31"/>
+      <c r="B65" s="31"/>
+      <c r="C65" s="41"/>
+      <c r="D65" s="41"/>
+      <c r="E65" s="41"/>
+      <c r="F65" s="41"/>
+      <c r="G65" s="41"/>
+      <c r="H65" s="41"/>
+      <c r="I65" s="41"/>
+      <c r="J65" s="41"/>
+      <c r="K65" s="41"/>
+      <c r="L65" s="41"/>
+      <c r="M65" s="41"/>
+      <c r="N65" s="41"/>
+      <c r="O65" s="41"/>
       <c r="P65" s="9"/>
-      <c r="Q65" s="28"/>
+      <c r="Q65" s="31"/>
     </row>
     <row r="66" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A66" s="28"/>
-      <c r="B66" s="28"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="9"/>
-      <c r="F66" s="9"/>
-      <c r="G66" s="9"/>
-      <c r="H66" s="9"/>
-      <c r="I66" s="9"/>
-      <c r="J66" s="9"/>
-      <c r="K66" s="9"/>
-      <c r="L66" s="9"/>
-      <c r="M66" s="9"/>
-      <c r="N66" s="9"/>
-      <c r="O66" s="9"/>
+      <c r="A66" s="31"/>
+      <c r="B66" s="31"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
+      <c r="E66" s="41"/>
+      <c r="F66" s="41"/>
+      <c r="G66" s="41"/>
+      <c r="H66" s="41"/>
+      <c r="I66" s="41"/>
+      <c r="J66" s="41"/>
+      <c r="K66" s="41"/>
+      <c r="L66" s="41"/>
+      <c r="M66" s="41"/>
+      <c r="N66" s="41"/>
+      <c r="O66" s="41"/>
       <c r="P66" s="9"/>
-      <c r="Q66" s="28"/>
+      <c r="Q66" s="31"/>
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A67" s="28"/>
-      <c r="B67" s="28"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="9"/>
-      <c r="F67" s="9"/>
-      <c r="G67" s="9"/>
-      <c r="H67" s="9"/>
-      <c r="I67" s="9"/>
-      <c r="J67" s="9"/>
-      <c r="K67" s="9"/>
-      <c r="L67" s="9"/>
-      <c r="M67" s="9"/>
-      <c r="N67" s="9"/>
-      <c r="O67" s="9"/>
+      <c r="A67" s="31"/>
+      <c r="B67" s="31"/>
+      <c r="C67" s="41"/>
+      <c r="D67" s="41"/>
+      <c r="E67" s="41"/>
+      <c r="F67" s="41"/>
+      <c r="G67" s="41"/>
+      <c r="H67" s="41"/>
+      <c r="I67" s="41"/>
+      <c r="J67" s="41"/>
+      <c r="K67" s="41"/>
+      <c r="L67" s="41"/>
+      <c r="M67" s="41"/>
+      <c r="N67" s="41"/>
+      <c r="O67" s="41"/>
       <c r="P67" s="9"/>
-      <c r="Q67" s="28"/>
+      <c r="Q67" s="31"/>
     </row>
     <row r="68" spans="1:17" ht="8.4499999999999993" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="28"/>
-      <c r="B68" s="28"/>
+      <c r="A68" s="31"/>
+      <c r="B68" s="31"/>
       <c r="C68" s="9"/>
       <c r="D68" s="9"/>
       <c r="E68" s="9"/>
@@ -2837,11 +2842,11 @@
       <c r="N68" s="9"/>
       <c r="O68" s="9"/>
       <c r="P68" s="9"/>
-      <c r="Q68" s="28"/>
+      <c r="Q68" s="31"/>
     </row>
     <row r="69" spans="1:17" ht="8.4499999999999993" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="28"/>
-      <c r="B69" s="28"/>
+      <c r="A69" s="31"/>
+      <c r="B69" s="31"/>
       <c r="C69" s="9"/>
       <c r="D69" s="9"/>
       <c r="E69" s="9"/>
@@ -2856,11 +2861,11 @@
       <c r="N69" s="9"/>
       <c r="O69" s="9"/>
       <c r="P69" s="9"/>
-      <c r="Q69" s="28"/>
+      <c r="Q69" s="31"/>
     </row>
     <row r="70" spans="1:17" ht="8.4499999999999993" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="28"/>
-      <c r="B70" s="28"/>
+      <c r="A70" s="31"/>
+      <c r="B70" s="31"/>
       <c r="C70" s="9"/>
       <c r="D70" s="9"/>
       <c r="E70" s="9"/>
@@ -2875,51 +2880,51 @@
       <c r="N70" s="9"/>
       <c r="O70" s="9"/>
       <c r="P70" s="9"/>
-      <c r="Q70" s="28"/>
+      <c r="Q70" s="31"/>
     </row>
     <row r="71" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="28"/>
-      <c r="B71" s="28"/>
-      <c r="C71" s="34" t="s">
+      <c r="A71" s="31"/>
+      <c r="B71" s="31"/>
+      <c r="C71" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="D71" s="34"/>
-      <c r="E71" s="34"/>
-      <c r="F71" s="34"/>
-      <c r="G71" s="34"/>
-      <c r="H71" s="28"/>
-      <c r="I71" s="28"/>
-      <c r="J71" s="28"/>
-      <c r="K71" s="28"/>
-      <c r="L71" s="28"/>
-      <c r="M71" s="28"/>
-      <c r="N71" s="28"/>
-      <c r="O71" s="28"/>
-      <c r="P71" s="28"/>
-      <c r="Q71" s="28"/>
+      <c r="D71" s="36"/>
+      <c r="E71" s="36"/>
+      <c r="F71" s="36"/>
+      <c r="G71" s="36"/>
+      <c r="H71" s="31"/>
+      <c r="I71" s="31"/>
+      <c r="J71" s="31"/>
+      <c r="K71" s="31"/>
+      <c r="L71" s="31"/>
+      <c r="M71" s="31"/>
+      <c r="N71" s="31"/>
+      <c r="O71" s="31"/>
+      <c r="P71" s="31"/>
+      <c r="Q71" s="31"/>
     </row>
     <row r="72" spans="1:17" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="28"/>
-      <c r="B72" s="28"/>
-      <c r="C72" s="28"/>
-      <c r="D72" s="28"/>
-      <c r="E72" s="28"/>
-      <c r="F72" s="28"/>
-      <c r="G72" s="28"/>
-      <c r="H72" s="28"/>
-      <c r="I72" s="28"/>
-      <c r="J72" s="28"/>
-      <c r="K72" s="28"/>
-      <c r="L72" s="28"/>
-      <c r="M72" s="28"/>
-      <c r="N72" s="28"/>
-      <c r="O72" s="28"/>
-      <c r="P72" s="28"/>
-      <c r="Q72" s="28"/>
+      <c r="A72" s="31"/>
+      <c r="B72" s="31"/>
+      <c r="C72" s="31"/>
+      <c r="D72" s="31"/>
+      <c r="E72" s="31"/>
+      <c r="F72" s="31"/>
+      <c r="G72" s="31"/>
+      <c r="H72" s="31"/>
+      <c r="I72" s="31"/>
+      <c r="J72" s="31"/>
+      <c r="K72" s="31"/>
+      <c r="L72" s="31"/>
+      <c r="M72" s="31"/>
+      <c r="N72" s="31"/>
+      <c r="O72" s="31"/>
+      <c r="P72" s="31"/>
+      <c r="Q72" s="31"/>
     </row>
     <row r="73" spans="1:17" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="28"/>
-      <c r="B73" s="28"/>
+      <c r="A73" s="31"/>
+      <c r="B73" s="31"/>
       <c r="C73" s="11"/>
       <c r="D73" s="11"/>
       <c r="E73" s="11"/>
@@ -2934,76 +2939,95 @@
       <c r="N73" s="11"/>
       <c r="O73" s="11"/>
       <c r="P73" s="11"/>
-      <c r="Q73" s="28"/>
+      <c r="Q73" s="31"/>
     </row>
     <row r="74" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A74" s="28"/>
-      <c r="B74" s="28"/>
+      <c r="A74" s="31"/>
+      <c r="B74" s="31"/>
       <c r="C74" s="7" t="s">
         <v>48</v>
       </c>
       <c r="D74" s="21"/>
       <c r="E74" s="22"/>
-      <c r="G74" s="28"/>
-      <c r="H74" s="28"/>
-      <c r="I74" s="28"/>
-      <c r="J74" s="28"/>
-      <c r="K74" s="28"/>
-      <c r="L74" s="28"/>
-      <c r="M74" s="28"/>
-      <c r="N74" s="32" t="s">
+      <c r="G74" s="31"/>
+      <c r="H74" s="31"/>
+      <c r="I74" s="31"/>
+      <c r="J74" s="31"/>
+      <c r="K74" s="31"/>
+      <c r="L74" s="31"/>
+      <c r="M74" s="31"/>
+      <c r="N74" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="O74" s="32"/>
-      <c r="P74" s="32"/>
-      <c r="Q74" s="28"/>
+      <c r="O74" s="34"/>
+      <c r="P74" s="34"/>
+      <c r="Q74" s="31"/>
     </row>
     <row r="75" spans="1:17" ht="13.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="28"/>
-      <c r="B75" s="28"/>
-      <c r="C75" s="28"/>
-      <c r="D75" s="28"/>
-      <c r="E75" s="28"/>
-      <c r="F75" s="28"/>
-      <c r="G75" s="28"/>
-      <c r="H75" s="28"/>
-      <c r="I75" s="28"/>
-      <c r="J75" s="28"/>
-      <c r="K75" s="28"/>
-      <c r="L75" s="28"/>
-      <c r="M75" s="28"/>
-      <c r="N75" s="28"/>
-      <c r="O75" s="28"/>
-      <c r="P75" s="28"/>
-      <c r="Q75" s="28"/>
+      <c r="A75" s="31"/>
+      <c r="B75" s="31"/>
+      <c r="C75" s="31"/>
+      <c r="D75" s="31"/>
+      <c r="E75" s="31"/>
+      <c r="F75" s="31"/>
+      <c r="G75" s="31"/>
+      <c r="H75" s="31"/>
+      <c r="I75" s="31"/>
+      <c r="J75" s="31"/>
+      <c r="K75" s="31"/>
+      <c r="L75" s="31"/>
+      <c r="M75" s="31"/>
+      <c r="N75" s="31"/>
+      <c r="O75" s="31"/>
+      <c r="P75" s="31"/>
+      <c r="Q75" s="31"/>
     </row>
     <row r="76" spans="1:17" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B76" s="28"/>
-      <c r="C76" s="28"/>
-      <c r="D76" s="28"/>
-      <c r="E76" s="28"/>
-      <c r="F76" s="28"/>
-      <c r="G76" s="28"/>
-      <c r="H76" s="28"/>
-      <c r="I76" s="28"/>
-      <c r="J76" s="28"/>
-      <c r="K76" s="28"/>
-      <c r="L76" s="28"/>
-      <c r="M76" s="28"/>
-      <c r="N76" s="28"/>
-      <c r="O76" s="28"/>
-      <c r="P76" s="28"/>
-      <c r="Q76" s="28"/>
+      <c r="B76" s="31"/>
+      <c r="C76" s="31"/>
+      <c r="D76" s="31"/>
+      <c r="E76" s="31"/>
+      <c r="F76" s="31"/>
+      <c r="G76" s="31"/>
+      <c r="H76" s="31"/>
+      <c r="I76" s="31"/>
+      <c r="J76" s="31"/>
+      <c r="K76" s="31"/>
+      <c r="L76" s="31"/>
+      <c r="M76" s="31"/>
+      <c r="N76" s="31"/>
+      <c r="O76" s="31"/>
+      <c r="P76" s="31"/>
+      <c r="Q76" s="31"/>
     </row>
   </sheetData>
-  <mergeCells count="48">
-    <mergeCell ref="F8:J8"/>
-    <mergeCell ref="F20:J20"/>
-    <mergeCell ref="F28:J28"/>
-    <mergeCell ref="F44:J44"/>
-    <mergeCell ref="C21:P21"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C28:D28"/>
+  <mergeCells count="49">
+    <mergeCell ref="C59:O67"/>
+    <mergeCell ref="C51:P51"/>
+    <mergeCell ref="L36:P40"/>
+    <mergeCell ref="C29:P29"/>
+    <mergeCell ref="C31:P31"/>
+    <mergeCell ref="L44:P46"/>
+    <mergeCell ref="C43:P43"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="O42:P42"/>
+    <mergeCell ref="L32:O32"/>
+    <mergeCell ref="B75:Q76"/>
+    <mergeCell ref="C47:P47"/>
+    <mergeCell ref="N74:P74"/>
+    <mergeCell ref="L52:P52"/>
+    <mergeCell ref="C71:G71"/>
+    <mergeCell ref="B2:B74"/>
+    <mergeCell ref="F12:J12"/>
+    <mergeCell ref="F16:J16"/>
+    <mergeCell ref="F18:J18"/>
+    <mergeCell ref="F10:J10"/>
+    <mergeCell ref="H26:N26"/>
+    <mergeCell ref="F34:J34"/>
+    <mergeCell ref="F38:J38"/>
+    <mergeCell ref="H50:M50"/>
+    <mergeCell ref="C5:P5"/>
+    <mergeCell ref="F52:J52"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="Q2:Q74"/>
     <mergeCell ref="L28:P28"/>
@@ -3020,31 +3044,13 @@
     <mergeCell ref="G74:M74"/>
     <mergeCell ref="A2:A75"/>
     <mergeCell ref="F6:J6"/>
-    <mergeCell ref="B75:Q76"/>
-    <mergeCell ref="C47:P47"/>
-    <mergeCell ref="N74:P74"/>
-    <mergeCell ref="L52:P52"/>
-    <mergeCell ref="C71:G71"/>
-    <mergeCell ref="B2:B74"/>
-    <mergeCell ref="F12:J12"/>
-    <mergeCell ref="F16:J16"/>
-    <mergeCell ref="F18:J18"/>
-    <mergeCell ref="F10:J10"/>
-    <mergeCell ref="H26:N26"/>
-    <mergeCell ref="F34:J34"/>
-    <mergeCell ref="F38:J38"/>
-    <mergeCell ref="H50:M50"/>
-    <mergeCell ref="C5:P5"/>
-    <mergeCell ref="F52:J52"/>
-    <mergeCell ref="C51:P51"/>
-    <mergeCell ref="L36:P40"/>
-    <mergeCell ref="C29:P29"/>
-    <mergeCell ref="C31:P31"/>
-    <mergeCell ref="L44:P46"/>
-    <mergeCell ref="C43:P43"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="O42:P42"/>
-    <mergeCell ref="L32:O32"/>
+    <mergeCell ref="F8:J8"/>
+    <mergeCell ref="F20:J20"/>
+    <mergeCell ref="F28:J28"/>
+    <mergeCell ref="F44:J44"/>
+    <mergeCell ref="C21:P21"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C28:D28"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="10001" scale="63" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>